<commit_message>
Ransomware feed update — 2026-05-07 08:22 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Conti, Akira ransomware affiliate given 8-year sentence - The Record from Recorded Future News</t>
+          <t>Iranian cyber espionage disguised as a Chaos Ransomware attack - Security Affairs</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 05 May 2026 17:40:45 GMT</t>
+          <t>Wed, 06 May 2026 14:34:20 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1QVnRFNVdjS1BJSGFuWHg3NXdXdXRtM3ZyamJpUTNocmctT1VHY0JkTjY3U1JPVTRkeldWWlVqNGM2WXdvOVVfdVdSVFk4OWUzMFZnX1I5M2RkbldVdXp4RDZpUElqcXgyS1lnelJYQUV2azR6?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQTFVxSlBCYkhLcUt6R2F5d3p5NTlvY0taX2ZEbTQ0RndxLVJfT1pMY3RWeWF1TF9CUTRXSHhsb2cySnp5YlFhQS1fMGk3TXVaMXBmVFd6NlpNalJUX1RqLTU0TWlkcTRSVmd1a05uNjhiNHdSNkt1LVlESlBsUDFJQ1J3NmVmUEZhdTNta24tM2l6ZS1MNXFwSnZzamZ6THFteGdRaExBbkthTHN6T1Bpdkc0MGRWYms?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Healthcare Firm Suffers Major Ransomware Attack, Personal and Medical Data of 169,017 People Now at Risk - The Daily Hodl</t>
+          <t>MuddyWater Uses Microsoft Teams to Steal Credentials in False Flag Ransomware Attack - The Hacker News</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 07:09:58 GMT</t>
+          <t>Wed, 06 May 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPV1A1YWRTRkFjYzh2STVhZTE5Qll6WWNwRGdNbllVODdQVU1yUXUwazFYSUZNeTI4ZkhmMkdwVmVnb19heEs0QnB0S2NxWUtXOGY4LXdMcS1TSVhLTzVISXpJSEE5S0lYcUo1WG1VaEluT3VWZlI3ellZZWZBUFhfUnNwSE9VWTgycHVMZ3Z6WDViMmlwQndqZTUwdC1PLUl1eXVfWmxHOUN4dGZZT1ZfdnlEN2syZUdXTmM4S0ZpekVPTVl4VGk2MHNoVW9yWTBJU3fSAdcBQVVfeXFMUHh1bVhpLVZqblRJejJ0UVNseXJSOEh1MktnWkNPMlZPUVpSTUxxUFh0SDB3a19pYkxiZXR5ZGl3OVhWNk12dFRtY1JZdmh2NGlHcmxXcmdpS0E2MVVXRVh1Z2VFck5OYS1kZjcyZWMzX3loX3ZMaDVXSnhIdkQ5M05tUlpEZXkzRTVMcEVPN1FKdTN1Q2UyY3A5OXM1cVJuZk4xT2laSEo0UXYxczVDOVp6T2VkMk40TE9yeFRyVERIRVJlSXN5cTdxOEJLY0g5SG5jaE1QVFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE5kNURveUh3MVVUNnZRS2pZV3FPQkpOV29hd29XajJyLUoyeEdNZndQb2ppMjVHVnpZLWFtWFRtTTlyX2ZnaHk5dnZnZE9NQ2hnNGJwTjR3c2x4VkdCeUxRajF0ZzBPQzhhN1ZNVXR1WWdhc01OdjRLRm5fTmxvZw?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Incransom Ransomware Attack on Childplace Family Services - DeXpose</t>
+          <t>Starr Insurance Discloses Ransomware Attack - The HIPAA Journal</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 00:19:54 GMT</t>
+          <t>Wed, 06 May 2026 13:43:13 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNaUh4SmdIc2M1UHVaNVNIU0FtWmlVeXZyYVpPZUExTjlzVUxhTlBWLW9ZZGhGOWwxeHRTS0ZrZldhbXdWTHZxYUdXTXNCMHhrRDhxelJWZnRWTWE0cGtCX0ppRXZlMkpqc2puZUVJV3IyOE9DazBhcW82YmhpUmdsdFFaMnZCMFBJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE81SDAxQ2t0Y0VUdWZIVXRIaVUzSEZBQm5Wc01wNWEtcF9fU0hfRDNucFNBdHBuNm9IYmlDN25nSXhlVTlmMXZTckIxQWV3NHFBRm5Hd2w2VFZYcDlMMjFFX2FvdlBVMXVsTFc0MXNQTXI?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Two ransomware gangs now claim Cushman &amp; Wakefield after Salesforce breach claim - Cybernews</t>
+          <t>National cat charity on the prowl for Shetland volunteers - Shetland Times</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 00:31:59 GMT</t>
+          <t>Wed, 06 May 2026 13:09:00 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOVS1nZUoyR3RmVkZkbk5mMFAxVDlTeWg3bWRDUjVYbDd5al9SeWNpLXZBVEowMGhaSWZ0QmdGNnRkU3RkMUtmMzdSM0x3Vjlnd2hjdnFZdE5pa3JfTEJOMW5aMWhLRkl1V2NxODZBNjZ2R0p5WWhBQlJjVlJjY3VWaU5NYmJ0QVdLX2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPdnJuMjFLUmtHMXZZSEtTX0Y5UVBGWkI4RDJvRXE1Y1NEVEF4dGs2Q2xxc2V3bk50TDNtZVZncVN6alVzXzJ5SGJHU2dEOFF3eXhhTFJjLVdmQ05WUV81d1hzcWN5bThLZUVrQldCOEFRMjNpZVhpRWJnc3JaVGlIejM2SHFhTnBRbGZxY0JGaGQ2UEdqazJzU2kwR1lEZUFnNE5RVw?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -596,27 +596,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ransomware_Response</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kash Patel skewers Nancy Guthrie case, says FBI has been 'kept out' - The Detroit News</t>
+          <t>Cactus Announces First Quarter 2026 Results - Quantisnow</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 02:40:00 GMT</t>
+          <t>Thu, 07 May 2026 03:41:15 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOWWE4VUhJMUZqbm5aa3Z4anItT2twcWRyZVRiNHgxV09EWVpfcHlfT0Jlbzg5RTd4M2lBV3lQanZsSmsyQ2RzNVpQNmo4VTBBVXhwMVFyYUtrbU1kNkZZSGFCNWRyVWhzdHQxZDdKVlAzQkwxZzNKR2xTbVBlcUtDR1JiNWtGUndRRFhZUnBScnFkc3JZcDd1S0pYSEpMOFgzMnFHQVF2RDVFNWtUUG1iemJXLWhESnVqQUV6SXRySXNkdWZ0M1hXNXVpbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQLUNZa2hsRlJoOE4xa19WemItd2pncEtzV0hlM282SFhWMmJvTTBYd3RXZGIwVjZjcVFZWUE0TTNnUkdRU3BtbkZvNlM5SWprWVA5QnZpTmhiR3Ffcll0WEF6aVV5WWJnTWpteDRMckR3SXNSSnJhdmJWek14M1lxTUJjZHZENEJ3NGc?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -631,27 +631,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ransomware_Response</t>
+          <t>Ransomware_Tactics_Threats</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rochester Police, FBI Boston Disrupt Drug and Gang Activity at Seasons Corner Market - New Bedford Guide</t>
+          <t>Autonomous agents are reshaping AI security - SiliconANGLE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tue, 05 May 2026 12:04:50 GMT</t>
+          <t>Wed, 06 May 2026 18:33:49 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQWDZISGpHYmZqUm5MVnRjN1BxOFNacTBjSUtmS283OEFka1RjRm5jWnhVdmtOSl9vTG00QU5zaURsM0F5S0U4MWozZjlCVm9BRlhFWGpyZnlGNXNMZ3M2ZUpuMUd0eDZ5X1VsUGNHMjV6RXNWdjAzdUJVeUVHTkR0RDRhVXpadlVhSmtBbkZ0TmtSU0tXTjNqZlFrZWVTakdkc3hhX2tJbXplZXk5N3JJdmxFNUhrRV9FTDAw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOX1VVNlJSdlo3VWZ3Nzk1Q3pCMV9weTE2alBBeWFpNE5KTWtFQlJHVG9Zd1pyOU5sZU9NM1ZNcGJ1dVVIbDYyV0ZfRnUxUFJiRlhROUdNQUR0OEpIMG5fcEtyMEpqYldnZ0c4cFF3bXl3SEhmNmN3YWQ1MmtHMnFDYmQtUFI0TkE5WmdIY0RfVnoyVUEyZE9ZVWlqaXNnQkFlSG1HUg?oc=5</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -666,27 +666,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ransomware_Tactics_Threats</t>
+          <t>Ransomware_Vulnerabilities</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fake SSA Emails Drive Venomous#Helper Phishing Campaign - Infosecurity Magazine</t>
+          <t>Critical Buffer Overflow Vulnerability in PAN-OS Exploited in-the-Wild - wiz.io</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tue, 05 May 2026 14:00:00 GMT</t>
+          <t>Wed, 06 May 2026 12:33:26 GMT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPdmRDWGZGUGtyVzBtM0U5MjZPMTdEMnRiRXliQWl3dnJZUVJ6Um9mWEg2QktzWTM2N2RodTVlNE15ckFuZEZtcFhGOWdMRUhkelVYbHV1VXREVWlBUnJ3a1Z6V3A1RFFlMXVKOTVheVN6cWxPaVhFa0hJWEd6UlpnMUdxZ0FhQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQOThjQzR2cXh2bVRWcEcwcHA2YWZGTTczUjc1dmlKQWtsRjVzZzRLRjJ1N2hzS2twbDhiejNhNDJlVi00UEZjSWZPcjZBRUZURGttMmgzemVVWExFUmY1OEJVQVB6RG52dWRiTkl5TkFZbFJZamxZOXVtYTc5M0VPNzhsbmhSVWF1UElPa2tUME42UHBfUFlR?oc=5</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -711,58 +711,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Critical Palo Alto Firewalls Vulnerability Exploited in the Wild to Gain Root Access - CyberSecurityNews</t>
+          <t>A critical Palo Alto PAN-OS zero-day is being exploited in the wild - CyberScoop</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 02:57:39 GMT</t>
+          <t>Wed, 06 May 2026 19:50:39 GMT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9FMVpjODlJa3cxYUE1T0pDeW9wTFRscDJ4X0h2UDhxNGJpZzZnaFNCX1BPTjNILTdLcEl4MzR6b081emMwRzhMbUNLcDlQck92cnlrZ0QwVS1BakU2X0N1ek9LTGpPN3VIUDJ6MEZnNW5tQldIODMzM0VFMnFsTTjSAYQBQVVfeXFMTWE4TjM4V3RBS1pzbGRXRFF0SEZvNDlRSnpnb0M5Zk0wRDJ1SkcwVjh4cFo1WWFWQmxEYUFFNEtVTXNvbjJKWHI4U2lYc0JuTnpBejBLdGRMWjF2dC1HSDFad0taWEdKc0xQMkp6S05MTmUxY0N3U3hyODhELXdIbDZDZUZN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQYVdGSDdxYnVzc0t2Uk5SUDJsVUlDNVgxQlVNdzI5SkluYWhBSlVPeDNkN2RTS1JCYm1Kd1dfTVdyazNCNl9WNVNEa2JJWjJlR1FSU1Buei1Yd0hWdHRrZ2U2VHZDMmpBWVdVaTh5WXRPTnphTUtDTzlLUnJrMzR0dWFLc2p4TUhNSlBRV3ROcU94OVZSeWc?oc=5</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ransomware_Vulnerabilities</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>AI-Powered Tools Accelerate Zero-Day Exploitation For Cybercriminals - cyberpress.org</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Wed, 06 May 2026 00:13:52 GMT</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE53SGZiNDllcmFuQ2xVNzNnMVFyZ3FJMWhNbGVrdGxsNmJZd2pOQmRmTkpKM3JmanRYZUtHUkpDT3pIeVhYeTh2V0VKcU4wOXlZdlRRMGhaTlZqMXM1SHVPTHFmb1JuOWs?oc=5</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-08 07:20 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Iranian cyber espionage disguised as a Chaos Ransomware attack - Security Affairs</t>
+          <t>The Canvas Hack Is a New Kind of Ransomware Debacle - WIRED</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 14:34:20 GMT</t>
+          <t>Fri, 08 May 2026 05:02:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQTFVxSlBCYkhLcUt6R2F5d3p5NTlvY0taX2ZEbTQ0RndxLVJfT1pMY3RWeWF1TF9CUTRXSHhsb2cySnp5YlFhQS1fMGk3TXVaMXBmVFd6NlpNalJUX1RqLTU0TWlkcTRSVmd1a05uNjhiNHdSNkt1LVlESlBsUDFJQ1J3NmVmUEZhdTNta24tM2l6ZS1MNXFwSnZzamZ6THFteGdRaExBbkthTHN6T1Bpdkc0MGRWYms?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQX0xFcmVYLTF0WHh2eTJsVlp0SnplSDd5RTZma05tUHdGNFpMOFZRZTIxc1pEOXpMSm9taWR5VnZ2OUh4QjZOZUVJRkVkWEpCaUM1MzNWTEpObXBwYVpvdWpwQlYxLTFnT2kxcEtCVzVJZVFBVTZUQ1g0S2xreXhwVmRR?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MuddyWater Uses Microsoft Teams to Steal Credentials in False Flag Ransomware Attack - The Hacker News</t>
+          <t>Canvas is down as ShinyHunters threatens to leak schools’ data - The Verge</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 13:00:00 GMT</t>
+          <t>Thu, 07 May 2026 21:29:27 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE5kNURveUh3MVVUNnZRS2pZV3FPQkpOV29hd29XajJyLUoyeEdNZndQb2ppMjVHVnpZLWFtWFRtTTlyX2ZnaHk5dnZnZE9NQ2hnNGJwTjR3c2x4VkdCeUxRajF0ZzBPQzhhN1ZNVXR1WWdhc01OdjRLRm5fTmxvZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5NbFBxc0I2NUtITnYySkRGZkFzS2x6ZXJGSFpfYW5BMVg0dDhacFBoMFdVOFpsWW40ZVBRSWtfNUtoNFdiQlhNdWNKWkgzREJJRFoyR1RxdDBKa3FsQ0RWSnp1VHpKYUpSdTBpTzJkNFo?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Starr Insurance Discloses Ransomware Attack - The HIPAA Journal</t>
+          <t>Canvas Online Learning Platform Disabled After Breach by Hackers - nytimes.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 13:43:13 GMT</t>
+          <t>Fri, 08 May 2026 06:16:00 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE81SDAxQ2t0Y0VUdWZIVXRIaVUzSEZBQm5Wc01wNWEtcF9fU0hfRDNucFNBdHBuNm9IYmlDN25nSXhlVTlmMXZTckIxQWV3NHFBRm5Hd2w2VFZYcDlMMjFFX2FvdlBVMXVsTFc0MXNQTXI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPYkVKaXAwWVMxYzZVU0gtSnJaZkFCLUhOWkJENjdmQ0licjI3QklrTmhhakphbzc4RlBETUlWR2J6U25QZmkwbVBFRmo1NTVtUWFRSFBCUDBEbmI2ZjFQajMxQXFWeDE1Xzc2dFdtWXgtVGJHNFI2UG5SWTgtSVozdGozbVV6cEE?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>National cat charity on the prowl for Shetland volunteers - Shetland Times</t>
+          <t>LBUSD, Cal State, LBCC grading platform hacked in apparent ransomware attack - Long Beach Post</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 13:09:00 GMT</t>
+          <t>Thu, 07 May 2026 22:24:59 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPdnJuMjFLUmtHMXZZSEtTX0Y5UVBGWkI4RDJvRXE1Y1NEVEF4dGs2Q2xxc2V3bk50TDNtZVZncVN6alVzXzJ5SGJHU2dEOFF3eXhhTFJjLVdmQ05WUV81d1hzcWN5bThLZUVrQldCOEFRMjNpZVhpRWJnc3JaVGlIejM2SHFhTnBRbGZxY0JGaGQ2UEdqazJzU2kwR1lEZUFnNE5RVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVE5hRmNKMVJJQkRwWnZBdldPSXBFZlhfdmx2TTMwOTZIbnJvRW1qY2pXTnR1Q3gxclhWeHNyTXFlMWlOSVFtMEluWE02Q3dXeTM3dENMQndYRHNKcHFBWjZ5djdsODBaa2VDQW9lY2Fucy1wQm5jMEFrZGk1WGtJREQtM29NYXlaUjV2U3ZCRlJLRmZwQVMtSjFleFpmUWZndWtuWVQybWFKNGs?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -596,27 +596,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Tactics_Threats</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cactus Announces First Quarter 2026 Results - Quantisnow</t>
+          <t>Scammers Exploit Disposable VoIP Numbers to Bypass Reputation Blocking - gbhackers.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 03:41:15 GMT</t>
+          <t>Thu, 07 May 2026 09:52:57 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQLUNZa2hsRlJoOE4xa19WemItd2pncEtzV0hlM282SFhWMmJvTTBYd3RXZGIwVjZjcVFZWUE0TTNnUkdRU3BtbkZvNlM5SWprWVA5QnZpTmhiR3Ffcll0WEF6aVV5WWJnTWpteDRMckR3SXNSSnJhdmJWek14M1lxTUJjZHZENEJ3NGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE1BUm1mYUYwLVRZdkJqUTRHemlEYzU3V092c2xpRWNzcGtXTHI0MV9DTnFCcEdHZVVzV0hpLWtJQXNXZldEMXYxZThOZURIeHFhMFBEcEpEQkRydjYxXy15dS1ObTRJUQ?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -631,103 +631,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ransomware_Tactics_Threats</t>
+          <t>Ransomware_Vulnerabilities</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Autonomous agents are reshaping AI security - SiliconANGLE</t>
+          <t>Ivanti customers confront yet another actively exploited zero-day - CyberScoop</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Wed, 06 May 2026 18:33:49 GMT</t>
+          <t>Thu, 07 May 2026 21:59:16 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOX1VVNlJSdlo3VWZ3Nzk1Q3pCMV9weTE2alBBeWFpNE5KTWtFQlJHVG9Zd1pyOU5sZU9NM1ZNcGJ1dVVIbDYyV0ZfRnUxUFJiRlhROUdNQUR0OEpIMG5fcEtyMEpqYldnZ0c4cFF3bXl3SEhmNmN3YWQ1MmtHMnFDYmQtUFI0TkE5WmdIY0RfVnoyVUEyZE9ZVWlqaXNnQkFlSG1HUg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5hajI0N3NVXzBmY3hHZzBjV21GaUZ4TC1vdy1jekNQdnVZbjV2VFJtRHM4Q0VzRUh1Wlg0ek40S2NNbkY0VXFabVktWFdiaklPZmFqT2czbmJBaVVsV3JRZXZWZVNmamVhMkNHellRbC1KdkxVVGJZ?oc=5</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ransomware_Vulnerabilities</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Critical Buffer Overflow Vulnerability in PAN-OS Exploited in-the-Wild - wiz.io</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Wed, 06 May 2026 12:33:26 GMT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQOThjQzR2cXh2bVRWcEcwcHA2YWZGTTczUjc1dmlKQWtsRjVzZzRLRjJ1N2hzS2twbDhiejNhNDJlVi00UEZjSWZPcjZBRUZURGttMmgzemVVWExFUmY1OEJVQVB6RG52dWRiTkl5TkFZbFJZamxZOXVtYTc5M0VPNzhsbmhSVWF1UElPa2tUME42UHBfUFlR?oc=5</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Ransomware_Vulnerabilities</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>A critical Palo Alto PAN-OS zero-day is being exploited in the wild - CyberScoop</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Wed, 06 May 2026 19:50:39 GMT</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQYVdGSDdxYnVzc0t2Uk5SUDJsVUlDNVgxQlVNdzI5SkluYWhBSlVPeDNkN2RTS1JCYm1Kd1dfTVdyazNCNl9WNVNEa2JJWjJlR1FSU1Buei1Yd0hWdHRrZ2U2VHZDMmpBWVdVaTh5WXRPTnphTUtDTzlLUnJrMzR0dWFLc2p4TUhNSlBRV3ROcU94OVZSeWc?oc=5</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-08 08:37 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Canvas is down as ShinyHunters threatens to leak schools’ data - The Verge</t>
+          <t>Canvas Online Learning Platform Shut Down for Hours After Cyberattack - nytimes.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 21:29:27 GMT</t>
+          <t>Fri, 08 May 2026 05:58:42 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5NbFBxc0I2NUtITnYySkRGZkFzS2x6ZXJGSFpfYW5BMVg0dDhacFBoMFdVOFpsWW40ZVBRSWtfNUtoNFdiQlhNdWNKWkgzREJJRFoyR1RxdDBKa3FsQ0RWSnp1VHpKYUpSdTBpTzJkNFo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPYkVKaXAwWVMxYzZVU0gtSnJaZkFCLUhOWkJENjdmQ0licjI3QklrTmhhakphbzc4RlBETUlWR2J6U25QZmkwbVBFRmo1NTVtUWFRSFBCUDBEbmI2ZjFQajMxQXFWeDE1Xzc2dFdtWXgtVGJHNFI2UG5SWTgtSVozdGozbVV6cEE?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Canvas Online Learning Platform Disabled After Breach by Hackers - nytimes.com</t>
+          <t>Canvas is down as ShinyHunters threatens to leak schools’ data - The Verge</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 06:16:00 GMT</t>
+          <t>Thu, 07 May 2026 21:29:27 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPYkVKaXAwWVMxYzZVU0gtSnJaZkFCLUhOWkJENjdmQ0licjI3QklrTmhhakphbzc4RlBETUlWR2J6U25QZmkwbVBFRmo1NTVtUWFRSFBCUDBEbmI2ZjFQajMxQXFWeDE1Xzc2dFdtWXgtVGJHNFI2UG5SWTgtSVozdGozbVV6cEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5NbFBxc0I2NUtITnYySkRGZkFzS2x6ZXJGSFpfYW5BMVg0dDhacFBoMFdVOFpsWW40ZVBRSWtfNUtoNFdiQlhNdWNKWkgzREJJRFoyR1RxdDBKa3FsQ0RWSnp1VHpKYUpSdTBpTzJkNFo?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-09 07:47 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The Canvas Hack Is a New Kind of Ransomware Debacle - WIRED</t>
+          <t>Starr Insurance discloses data breach following cyberattack claimed by Akira ransomware group - teiss</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 05:02:00 GMT</t>
+          <t>Fri, 08 May 2026 14:10:05 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQX0xFcmVYLTF0WHh2eTJsVlp0SnplSDd5RTZma05tUHdGNFpMOFZRZTIxc1pEOXpMSm9taWR5VnZ2OUh4QjZOZUVJRkVkWEpCaUM1MzNWTEpObXBwYVpvdWpwQlYxLTFnT2kxcEtCVzVJZVFBVTZUQ1g0S2xreXhwVmRR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxORXdHWm9CZ0ota0drRllvaDczUG42TlUzS3F0N3hlQkVaNUtXSTJEalQwal80UlJkd0lEekhTNlJJTmQ0SXh0d251em9zN09LNFlDQmVBRG1LNE1md04zWl9EZXN6NTFXUzh3YUlCMFZiY0oxOFFGS3Jzb1lTLUtDNjJEa0tlQ1lKcFo3Y2hyRWgySWlPSl9oclZGcjdZcU5weWRYZlNOZXF0MTBGdkIyQ2ZHOUZzRXBLR2ZMUmc3NE40RVhkc1dV?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Canvas Online Learning Platform Shut Down for Hours After Cyberattack - nytimes.com</t>
+          <t>Canvas returns after ShinyHunters ransomware attack on Instructure - - The Mercer Cluster</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 05:58:42 GMT</t>
+          <t>Fri, 08 May 2026 13:29:00 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPYkVKaXAwWVMxYzZVU0gtSnJaZkFCLUhOWkJENjdmQ0licjI3QklrTmhhakphbzc4RlBETUlWR2J6U25QZmkwbVBFRmo1NTVtUWFRSFBCUDBEbmI2ZjFQajMxQXFWeDE1Xzc2dFdtWXgtVGJHNFI2UG5SWTgtSVozdGozbVV6cEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNRmU5R2VPb0VmWjBSbnBjSHZaSlBHNFFWOGdmLVpYamtaanVuSm9KVTNOY3FDdlB6N192NWN0Ty1KM2NvYjZZOEJSWmViVUQ3bmhyY3V2b0gyVVQ3cndvc3JwdFZPaWhpNjRsY0ZfRUtwWENzSGV5UDA1R0tJYjV6SzBBOVlaR28?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Canvas is down as ShinyHunters threatens to leak schools’ data - The Verge</t>
+          <t>Maryland school districts, colleges shut down Canvas amid ransomware attack - WBAL-TV</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 21:29:27 GMT</t>
+          <t>Fri, 08 May 2026 22:15:00 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5NbFBxc0I2NUtITnYySkRGZkFzS2x6ZXJGSFpfYW5BMVg0dDhacFBoMFdVOFpsWW40ZVBRSWtfNUtoNFdiQlhNdWNKWkgzREJJRFoyR1RxdDBKa3FsQ0RWSnp1VHpKYUpSdTBpTzJkNFo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNZVdGUUZuUmFsaFNFUmtFbXFSVTFIQ3JkNkJLbHBCaTAta2syV1hDQUxmVEVNcHkwVndHZWhaUWJjMm8yNWpIbDk1MndXbnVJWmo0dkhRdGVkMVBTbG5MamJad3VSYzczZFRrOVpQUnhMV0lKNjRKM0FZVkR3MkpydERvOERDTm8tODNDVXZmby0wOGdZ?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Incidents_UK_EU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>(ransomware OR "cyber attack" OR "data breach") AND (NHS OR "local council" OR "local authority" OR "public sector" OR university OR school OR manufacturer OR retailer OR "law firm") AND (UK OR Britain OR England OR Scotland OR Wales OR Ireland OR Germany OR France OR Italy OR Spain OR Europe)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LBUSD, Cal State, LBCC grading platform hacked in apparent ransomware attack - Long Beach Post</t>
+          <t>International cyber attack disrupts swathe of universities and schools - BBC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 22:24:59 GMT</t>
+          <t>Fri, 08 May 2026 12:27:02 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVE5hRmNKMVJJQkRwWnZBdldPSXBFZlhfdmx2TTMwOTZIbnJvRW1qY2pXTnR1Q3gxclhWeHNyTXFlMWlOSVFtMEluWE02Q3dXeTM3dENMQndYRHNKcHFBWjZ5djdsODBaa2VDQW9lY2Fucy1wQm5jMEFrZGk1WGtJREQtM29NYXlaUjV2U3ZCRlJLRmZwQVMtSjFleFpmUWZndWtuWVQybWFKNGs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5lUlcyLU9pbFpJTnlSZ3MycmFWeFdFQnZHZFJnZmVKUGUwR0VoOEpScFpjOTlTMFdNQm5JNVV5QXRsblJPaDg3bEdyMFdQZ041aWpKMUN2NjBLS3Jv?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -596,68 +596,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ransomware_Tactics_Threats</t>
+          <t>Ransomware_Response</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Scammers Exploit Disposable VoIP Numbers to Bypass Reputation Blocking - gbhackers.com</t>
+          <t>FBI Seeks Tips On Danny Liggett, Wanted For A 1987 Murder In Manhattan - 101.5 WPDH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thu, 07 May 2026 09:52:57 GMT</t>
+          <t>Fri, 08 May 2026 13:12:07 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE1BUm1mYUYwLVRZdkJqUTRHemlEYzU3V092c2xpRWNzcGtXTHI0MV9DTnFCcEdHZVVzV0hpLWtJQXNXZldEMXYxZThOZURIeHFhMFBEcEpEQkRydjYxXy15dS1ObTRJUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE1LMXBZc1VqZERPcnF1SmxIbDktNmpSNXhGUUpWOGh1endyNHRZMXhTdHVaZW4tMzVQS1ZVbXpxTnUxMnZOYVZlTlcwdEJfVlI0RkNIdA?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ransomware_Vulnerabilities</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ivanti customers confront yet another actively exploited zero-day - CyberScoop</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Thu, 07 May 2026 21:59:16 GMT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5hajI0N3NVXzBmY3hHZzBjV21GaUZ4TC1vdy1jekNQdnVZbjV2VFJtRHM4Q0VzRUh1Wlg0ek40S2NNbkY0VXFabVktWFdiaklPZmFqT2czbmJBaVVsV3JRZXZWZVNmamVhMkNHellRbC1KdkxVVGJZ?oc=5</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-10 08:01 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Starr Insurance discloses data breach following cyberattack claimed by Akira ransomware group - teiss</t>
+          <t>U of I restores access to the Canvas learning platform following ransomware attack - IPM Newsroom</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 14:10:05 GMT</t>
+          <t>Sat, 09 May 2026 21:19:26 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxORXdHWm9CZ0ota0drRllvaDczUG42TlUzS3F0N3hlQkVaNUtXSTJEalQwal80UlJkd0lEekhTNlJJTmQ0SXh0d251em9zN09LNFlDQmVBRG1LNE1md04zWl9EZXN6NTFXUzh3YUlCMFZiY0oxOFFGS3Jzb1lTLUtDNjJEa0tlQ1lKcFo3Y2hyRWgySWlPSl9oclZGcjdZcU5weWRYZlNOZXF0MTBGdkIyQ2ZHOUZzRXBLR2ZMUmc3NE40RVhkc1dV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOV1FwaDZ5Q3R0RzRCSEJlOUpFeTNqNVlqYV9vMUxZYVY4bUFRcV9MVlVxdFNNQXdCMzMwZGl4NzR6RUpETWdVZnZGUHRMTXVkSGZVcEt5Y2JoR19fajFVaUJCYUZqTS1jYTdhMy1MSFNHV05mc19QdU5Fa29RR296SXVuclcyWkFkSTZRMExVbENYeks3NHdMV29JZldhSm9ES2h0WG5aWkVOQQ?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Canvas returns after ShinyHunters ransomware attack on Instructure - - The Mercer Cluster</t>
+          <t>Lamashtu Strikes Ashtech Infotech with Ransomware Attack - DeXpose</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 13:29:00 GMT</t>
+          <t>Sun, 10 May 2026 06:48:08 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNRmU5R2VPb0VmWjBSbnBjSHZaSlBHNFFWOGdmLVpYamtaanVuSm9KVTNOY3FDdlB6N192NWN0Ty1KM2NvYjZZOEJSWmViVUQ3bmhyY3V2b0gyVVQ3cndvc3JwdFZPaWhpNjRsY0ZfRUtwWENzSGV5UDA1R0tJYjV6SzBBOVlaR28?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOdUxLNGpZdmZCWHVWT0JQRWZZbmtZSUFreTVxdjdZNVZEZmV0MW5Idl8xY09Lb1VFdC1FaWJVZUM3VW1wbnp1eUVqYjRkMXJSWUJyTlhUR3BJNTdHWkEwaGZSYy1NejVPdGdKN1VuYi02UGJ4NXE2Q1dMVVBmX25rZW1JSFVDYWc?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Maryland school districts, colleges shut down Canvas amid ransomware attack - WBAL-TV</t>
+          <t>Ransomware attack wipes out finals week at ISU, thousands of other schools - Idaho State Journal</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 22:15:00 GMT</t>
+          <t>Sat, 09 May 2026 19:28:00 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNZVdGUUZuUmFsaFNFUmtFbXFSVTFIQ3JkNkJLbHBCaTAta2syV1hDQUxmVEVNcHkwVndHZWhaUWJjMm8yNWpIbDk1MndXbnVJWmo0dkhRdGVkMVBTbG5MamJad3VSYzczZFRrOVpQUnhMV0lKNjRKM0FZVkR3MkpydERvOERDTm8tODNDVXZmby0wOGdZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOWG14eF9VdElfRjNFRExQaWw0dU5hYVp0dnZmc1pYSlhlVFZqcmlvdC1pZlB2aXlKX08tcVUyWnN6WjFEVE5ULWFvcThMVENhM2lIdmlMbFp3em9fRFNET2w4ZTA2dEJVOVhlMXRvbXl2ZjdTcmFLVU9ncGJkMC1MVTNveDctVVQ2c0VseklNbDBEZ3BqeVB5aWtxOTBYRGMwYXlXWV8zSVZ4UUtDY3U1czdHTUY5OGJaUnFncl9UbFdOUi1KYlVNM3dzQ1FabzdGZ2NpcDN0b2lPVHJjX1pEcEFZV2dHUnZtMUxuSXVaODNNOGxnaHFfNmdpaFbSAYICQVVfeXFMUE84WmxjcVV5dU5aQy1ObHR2T1hYcUhCeFFOb3NDR21qWUV6cldRay1OQXZGS0p2cWc4eC1KVkYtWTZFVmdPcks0OVRIM3VYWFVFbWZ5U1RqUl9WcDhGR0VPelFVX045MHl6emVVbG5ZS0VsbHVURmo3MUxnY19DeVo0UDJuc0JrRHJpLUcwT3U5c1dRNXE2ZEMwOTY3VUpHY0FfYTl4Y2RubGdSVy1qY19oaWNRYnFIMXBJNkNtVHg1TlRuNHVtYURFb215RFJZcXJXQzF1T19ROUN2ajAzWFBBMG1ud0U3Z093ZHlqQWpmRVFGWVNkTUJrczByTEtNdnBB?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,68 +561,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Incidents_UK_EU</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(ransomware OR "cyber attack" OR "data breach") AND (NHS OR "local council" OR "local authority" OR "public sector" OR university OR school OR manufacturer OR retailer OR "law firm") AND (UK OR Britain OR England OR Scotland OR Wales OR Ireland OR Germany OR France OR Italy OR Spain OR Europe)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>International cyber attack disrupts swathe of universities and schools - BBC</t>
+          <t>UAE weather update: Humidity, fog and winds expected this week - Gulf News</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 12:27:02 GMT</t>
+          <t>Sat, 09 May 2026 20:00:32 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5lUlcyLU9pbFpJTnlSZ3MycmFWeFdFQnZHZFJnZmVKUGUwR0VoOEpScFpjOTlTMFdNQm5JNVV5QXRsblJPaDg3bEdyMFdQZ041aWpKMUN2NjBLS3Jv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNN1l3eWttNzhGOTBfOURiUndkS1Nnb2tRLWlHYlFxYUkyRy0zNGRGNFVTdTBoS1l5U09Rbm9vWWJuV1hpd0JYRlZkYmIzdzZnUW5HYW93cVZhc3ZCU0ZwYTYtT1JFRFVVRGR1RE5NNEdMaUZjTW9QQkNIZ3YzejZqYVpVRHI4VGxYZ25GWU5xazZKaUp5S3paN1pVeFVoRE94RnRuSDhnYjPSAbsBQVVfeXFMUF9SYXktWFJZVmtQQ2F2Wk1EN3dwNm10YjIxRU1QTEE5NmxUVWpBUWN5dFdGTGtaRGJPMzZ5b01ZQmZQTlpJeGo1Y1o2NmItTzZfd0ppQU5CbFo5b3BqQ2lWRkNXN1NCUjNxTnpUVVJZYjg2Uzd4SWFHak9qM1plcW82cjlCNWRrOWswZjZRUGVvLTkyNFB0OGJfM2ZQMlJiLWNkQWRTV0VOaW5yblNnQmRzZHNnVHEtT1lRUQ?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ransomware_Response</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>FBI Seeks Tips On Danny Liggett, Wanted For A 1987 Murder In Manhattan - 101.5 WPDH</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Fri, 08 May 2026 13:12:07 GMT</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE1LMXBZc1VqZERPcnF1SmxIbDktNmpSNXhGUUpWOGh1endyNHRZMXhTdHVaZW4tMzVQS1ZVbXpxTnUxMnZOYVZlTlcwdEJfVlI0RkNIdA?oc=5</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-11 09:29 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,146 +450,6 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>source</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ransomware_Activity</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>U of I restores access to the Canvas learning platform following ransomware attack - IPM Newsroom</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sat, 09 May 2026 21:19:26 GMT</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOV1FwaDZ5Q3R0RzRCSEJlOUpFeTNqNVlqYV9vMUxZYVY4bUFRcV9MVlVxdFNNQXdCMzMwZGl4NzR6RUpETWdVZnZGUHRMTXVkSGZVcEt5Y2JoR19fajFVaUJCYUZqTS1jYTdhMy1MSFNHV05mc19QdU5Fa29RR296SXVuclcyWkFkSTZRMExVbENYeks3NHdMV29JZldhSm9ES2h0WG5aWkVOQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ransomware_Activity</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Lamashtu Strikes Ashtech Infotech with Ransomware Attack - DeXpose</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sun, 10 May 2026 06:48:08 GMT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOdUxLNGpZdmZCWHVWT0JQRWZZbmtZSUFreTVxdjdZNVZEZmV0MW5Idl8xY09Lb1VFdC1FaWJVZUM3VW1wbnp1eUVqYjRkMXJSWUJyTlhUR3BJNTdHWkEwaGZSYy1NejVPdGdKN1VuYi02UGJ4NXE2Q1dMVVBmX25rZW1JSFVDYWc?oc=5</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ransomware_Activity</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Ransomware attack wipes out finals week at ISU, thousands of other schools - Idaho State Journal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sat, 09 May 2026 19:28:00 GMT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxOWG14eF9VdElfRjNFRExQaWw0dU5hYVp0dnZmc1pYSlhlVFZqcmlvdC1pZlB2aXlKX08tcVUyWnN6WjFEVE5ULWFvcThMVENhM2lIdmlMbFp3em9fRFNET2w4ZTA2dEJVOVhlMXRvbXl2ZjdTcmFLVU9ncGJkMC1MVTNveDctVVQ2c0VseklNbDBEZ3BqeVB5aWtxOTBYRGMwYXlXWV8zSVZ4UUtDY3U1czdHTUY5OGJaUnFncl9UbFdOUi1KYlVNM3dzQ1FabzdGZ2NpcDN0b2lPVHJjX1pEcEFZV2dHUnZtMUxuSXVaODNNOGxnaHFfNmdpaFbSAYICQVVfeXFMUE84WmxjcVV5dU5aQy1ObHR2T1hYcUhCeFFOb3NDR21qWUV6cldRay1OQXZGS0p2cWc4eC1KVkYtWTZFVmdPcks0OVRIM3VYWFVFbWZ5U1RqUl9WcDhGR0VPelFVX045MHl6emVVbG5ZS0VsbHVURmo3MUxnY19DeVo0UDJuc0JrRHJpLUcwT3U5c1dRNXE2ZEMwOTY3VUpHY0FfYTl4Y2RubGdSVy1qY19oaWNRYnFIMXBJNkNtVHg1TlRuNHVtYURFb215RFJZcXJXQzF1T19ROUN2ajAzWFBBMG1ud0U3Z093ZHlqQWpmRVFGWVNkTUJrczByTEtNdnBB?oc=5</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ransomware_Groups_New</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>UAE weather update: Humidity, fog and winds expected this week - Gulf News</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Sat, 09 May 2026 20:00:32 GMT</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNN1l3eWttNzhGOTBfOURiUndkS1Nnb2tRLWlHYlFxYUkyRy0zNGRGNFVTdTBoS1l5U09Rbm9vWWJuV1hpd0JYRlZkYmIzdzZnUW5HYW93cVZhc3ZCU0ZwYTYtT1JFRFVVRGR1RE5NNEdMaUZjTW9QQkNIZ3YzejZqYVpVRHI4VGxYZ25GWU5xazZKaUp5S3paN1pVeFVoRE94RnRuSDhnYjPSAbsBQVVfeXFMUF9SYXktWFJZVmtQQ2F2Wk1EN3dwNm10YjIxRU1QTEE5NmxUVWpBUWN5dFdGTGtaRGJPMzZ5b01ZQmZQTlpJeGo1Y1o2NmItTzZfd0ppQU5CbFo5b3BqQ2lWRkNXN1NCUjNxTnpUVVJZYjg2Uzd4SWFHak9qM1plcW82cjlCNWRrOWswZjZRUGVvLTkyNFB0OGJfM2ZQMlJiLWNkQWRTV0VOaW5yblNnQmRzZHNnVHEtT1lRUQ?oc=5</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>google_rss</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-11 11:51 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +453,1511 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>International cyber attack disrupts swathe of universities and schools - BBC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 01:17:55 GMT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFAxZW9KSEdtMm1maTdXV181LVdFTWhUUElaMWhrd19KTUpTdW5wVXRBNmlPbXl6QkgwRjJlcW5HMFFLR01ZRTBXOXBCdml3UXpzMVNyQ09tcGlyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Millions of students’ personal data stolen in major education breach - Malwarebytes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 13:00:25 GMT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOYnlDUU1uWjQzUmRtZDlpLUJjZXdrQVRkNG44ekthTTNZY1RjS2JpQzJuVzhiUk02aVd6S2I4blVGYnRUSVowRlJUMUw2LXc3X0ZvN0JnaEVtMWVrRVBQbnVhU3laWHpCMGVmLW96X3l6RWJ6VWhUSklfcG1Ed0p1QVI3N3p2aE1jVkdENl9CTDZsUWV5c2FWYThlRmcxV2VCMXcxS19Ua3ZTUjhOa1p5OXRtZXVwVV9naEtR?oc=5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The Canvas Hack Is a New Kind of Ransomware Debacle - WIRED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fri, 08 May 2026 05:02:00 GMT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQX0xFcmVYLTF0WHh2eTJsVlp0SnplSDd5RTZma05tUHdGNFpMOFZRZTIxc1pEOXpMSm9taWR5VnZ2OUh4QjZOZUVJRkVkWEpCaUM1MzNWTEpObXBwYVpvdWpwQlYxLTFnT2kxcEtCVzVJZVFBVTZUQ1g0S2xreXhwVmRR?oc=5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Education Sector in the Crosshairs: ShinyHunters' Extortion Campaign Against Instructure - Halcyon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 01:13:11 GMT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOX2xBUGdDOHBOMno4Q3F0VThjR3JQZDg0TzdJRFhlY2NjMUVSVzVFcXdSZzlNZGNnMkdOc3hLTUU1UWY3UExYcjhrZTVSWU1INWs1cVZyWGNhd0JjTmZaUEhNS0JHbmpvaVZiNnFtRF9XZjd1ZGx4MFpwMWFwdy1VSDBXRmZHaTlGcXBzcjRka2RsbXZqUHB0SHBialB4bmd3MDdwUEI3OHhEUGZzTE1tTVdUZ3RMbVBfNlIxUFlYdU5qQ243bFE?oc=5</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Iranian cyber espionage disguised as a Chaos Ransomware attack - Security Affairs</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 14:34:20 GMT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQTFVxSlBCYkhLcUt6R2F5d3p5NTlvY0taX2ZEbTQ0RndxLVJfT1pMY3RWeWF1TF9CUTRXSHhsb2cySnp5YlFhQS1fMGk3TXVaMXBmVFd6NlpNalJUX1RqLTU0TWlkcTRSVmd1a05uNjhiNHdSNkt1LVlESlBsUDFJQ1J3NmVmUEZhdTNta24tM2l6ZS1MNXFwSnZzamZ6THFteGdRaExBbkthTHN6T1Bpdkc0MGRWYms?oc=5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Conti, Akira ransomware affiliate given 8-year sentence - The Record from Recorded Future News</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tue, 05 May 2026 17:40:45 GMT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1QVnRFNVdjS1BJSGFuWHg3NXdXdXRtM3ZyamJpUTNocmctT1VHY0JkTjY3U1JPVTRkeldWWlVqNGM2WXdvOVVfdVdSVFk4OWUzMFZnX1I5M2RkbldVdXp4RDZpUElqcXgyS1lnelJYQUV2azR6?oc=5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Canvas is online again after ShinyHunters threaten to leak schools’ data - The Verge</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 21:29:27 GMT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5NbFBxc0I2NUtITnYySkRGZkFzS2x6ZXJGSFpfYW5BMVg0dDhacFBoMFdVOFpsWW40ZVBRSWtfNUtoNFdiQlhNdWNKWkgzREJJRFoyR1RxdDBKa3FsQ0RWSnp1VHpKYUpSdTBpTzJkNFo?oc=5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>“PAY OR LEAK”: Hackers Target Big Higher Ed Vendor - Inside Higher Ed</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tue, 05 May 2026 22:39:01 GMT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOdV9iUXJTQXIzMWJEX1VDZ2d2Wl8xdFk2cS1GbE83TnJicTlNQjVNNlBCZWZNeTF0SUNqU0hfenZJa1h4NVZ5djl1XzVpTXRtTENRdDB1TWtiNzk2OEIyLWdhdV9OTVlrTl9sWmphR2t0b0tiS1Y0YmhSVDhLRkdhN2FJbWRvNjg3bzVEVTd0bWd2RzVUNlFULU9QczJ2VUNidkRRc2xSQWFmdUNtNVZtMS05bjlzUTNvQ01DcGJNY0UxdW9DMVRqbTJn?oc=5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>30</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MuddyWater Uses Microsoft Teams to Steal Credentials in False Flag Ransomware Attack - The Hacker News</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 13:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE5kNURveUh3MVVUNnZRS2pZV3FPQkpOV29hd29XajJyLUoyeEdNZndQb2ppMjVHVnpZLWFtWFRtTTlyX2ZnaHk5dnZnZE9NQ2hnNGJwTjR3c2x4VkdCeUxRajF0ZzBPQzhhN1ZNVXR1WWdhc01OdjRLRm5fTmxvZw?oc=5</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>30</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LBUSD, Cal State, LBCC grading platform hacked in apparent ransomware attack - Long Beach Post</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 22:24:59 GMT</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPVE5hRmNKMVJJQkRwWnZBdldPSXBFZlhfdmx2TTMwOTZIbnJvRW1qY2pXTnR1Q3gxclhWeHNyTXFlMWlOSVFtMEluWE02Q3dXeTM3dENMQndYRHNKcHFBWjZ5djdsODBaa2VDQW9lY2Fucy1wQm5jMEFrZGk1WGtJREQtM29NYXlaUjV2U3ZCRlJLRmZwQVMtSjFleFpmUWZndWtuWVQybWFKNGs?oc=5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ransomware_Critical_Infra</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>(ransomware OR "cyber attack") AND ("critical infrastructure" OR "energy sector" OR "power grid" OR "water utility" OR "transport network" OR "financial services" OR "telecoms" OR "government systems") AND (attacked OR disrupted OR warning OR incident OR threat OR advisory)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FBI: Ransomware Still a Top Threat to Critical Infrastructure - govtech.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tue, 14 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOSUhybUlLNXB5dHhEVk0wcmJrSktzaElfNUQ3MWZzRTFFbVBXM0Y5ZFd3X3lZZ1FQODZnVmtGXzFQTTAyRVBmU3dFMnRHQlUzRDZiS0phY3JndWhTR1lYWExTcHNFaTBFZzB5bzdVaVhWLVM2OXkxOE1SYi1zMmhPWXdfd2gtSEdFVFE5STNOTF9STC16cFBvbQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>National cat charity on the prowl for Shetland volunteers - Shetland Times</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 13:09:00 GMT</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPdnJuMjFLUmtHMXZZSEtTX0Y5UVBGWkI4RDJvRXE1Y1NEVEF4dGs2Q2xxc2V3bk50TDNtZVZncVN6alVzXzJ5SGJHU2dEOFF3eXhhTFJjLVdmQ05WUV81d1hzcWN5bThLZUVrQldCOEFRMjNpZVhpRWJnc3JaVGlIejM2SHFhTnBRbGZxY0JGaGQ2UEdqazJzU2kwR1lEZUFnNE5RVw?oc=5</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>US Cuba embargo 'crosses the line under international law' - University of Reading</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Fri, 01 May 2026 10:43:36 GMT</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQREl5VUN5d0dDZExjYkFlN1pTcDNUVWFRb3g2REVURTh1Nkw0TFBEN2hHXzh3eEtEOFlOSkhSLWtsVXI3U3R4Um5Gd2ZWeEM5ekh1VUhmcjM5S0pzWnpYODRoc21CcFg0RGFyV1ExX05JcW80NFlYeWxaTjNWWjlaS0oxQ3J3ZG9n?oc=5</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>30</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>You May Have Never Heard of a Fishbone Cactus – But This Quirky, Low-Maintenance Houseplant is Surprisingly Easy to Grow - Homes and Gardens</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sun, 26 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE55UFZYZXphbEpqMlhZX3VKM3JidDM2OW43MEo4MlRYQzFnLW4xeFVrVmhyRG5BZldJT0JrZGsta2hnWkNxa21ObkpOUFZzQy13cWlkTWFYTDB5cW10enZuRXVTXzNpRUFybzBMZGhuZkJJenR1VktkSkNheldLQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cactus Announces First Quarter 2026 Results - Quantisnow</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 03:41:15 GMT</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQLUNZa2hsRlJoOE4xa19WemItd2pncEtzV0hlM282SFhWMmJvTTBYd3RXZGIwVjZjcVFZWUE0TTNnUkdRU3BtbkZvNlM5SWprWVA5QnZpTmhiR3Ffcll0WEF6aVV5WWJnTWpteDRMckR3SXNSSnJhdmJWek14M1lxTUJjZHZENEJ3NGc?oc=5</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>UAE weather update: Humidity, fog and winds expected this week - Gulf News</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 20:00:32 GMT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNN1l3eWttNzhGOTBfOURiUndkS1Nnb2tRLWlHYlFxYUkyRy0zNGRGNFVTdTBoS1l5U09Rbm9vWWJuV1hpd0JYRlZkYmIzdzZnUW5HYW93cVZhc3ZCU0ZwYTYtT1JFRFVVRGR1RE5NNEdMaUZjTW9QQkNIZ3YzejZqYVpVRHI4VGxYZ25GWU5xazZKaUp5S3paN1pVeFVoRE94RnRuSDhnYjPSAbsBQVVfeXFMUF9SYXktWFJZVmtQQ2F2Wk1EN3dwNm10YjIxRU1QTEE5NmxUVWpBUWN5dFdGTGtaRGJPMzZ5b01ZQmZQTlpJeGo1Y1o2NmItTzZfd0ppQU5CbFo5b3BqQ2lWRkNXN1NCUjNxTnpUVVJZYjg2Uzd4SWFHak9qM1plcW82cjlCNWRrOWswZjZRUGVvLTkyNFB0OGJfM2ZQMlJiLWNkQWRTV0VOaW5yblNnQmRzZHNnVHEtT1lRUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Real estate giant Cushman &amp; Wakefield confirms cyber incident, Qilin and ShinyHunters claim attack - Cyber Daily</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 00:43:14 GMT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNbzhKTVdFSEJNZ1JUY3pCZmpqUXZBX2lnWGtVcWk4S0NWQk1XVGIyN3c1dVFZYS0wUXVlVTRIMTEzYlNocVk1Vy1qSmN2N2pYZjFjemdmVDBaV1l0ZVNjQzZocXVBeWtaejVOVnVSQ09mVkViY3h6UW5adWoxandmelFUaGd2UDl6dmEtLWpGQmY5a0tfd3h6R2o5OGttOXo1bHVZSVE1V01rLUxLRkI0MEJkb2tiTFVva045RkhOaG4zMnNIU09kc3QyMXVSRU9fbVE?oc=5</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>30</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lynx - Carnivore, Solitary, Fur - Britannica</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Fri, 24 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1iUDI3d3JOTDRnam5MZUtIOGZJMmdGTjh3Rk1NVDM5clFKcDRBVnRnZVRPS0dITGNvS2NpYzA2VmxFdmdWbUtVRklITlhZVEI4aVU0d0NBdUhXVENRNjV3VFo0QTFVYWhWNERN?oc=5</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>30</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>“Seeing clearly even in the fog”: DGIST develops next-generation infrared image sensor for autonomous driving - EurekAlert!</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Mon, 20 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1EZVZ0T1hpYTNqTzdVV3lIcy1QbnRtNms0TjdtcW12RmZ3SGp5Q29mTFNGcUJIanBPcnlwLVNZYWxrTVo5R1VQNklYLWgwR0JteEdqQjZjcGlUSHVU?oc=5</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Is it brain fog or something more? The signs women shouldn’t ignore - The Australian Women's Weekly</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tue, 28 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBLemFHNk1PUEVhTWkyWEgyZDVzQTZUZTk4ZjFDLTB0S3gwVENyVS1IZF85NFhQNUx6YlVKX2VubjNQQTd0V3dIY2xJcU81VHYzTktycDZDVm4td3hyUFpheW41WnZiUHVsdHpLb01B?oc=5</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>30</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>What women need to know about brain fog and perimenopause - Glamour South Africa</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mon, 20 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQS1lnYlBsZDlqUXBwYlY5Z2toYUZNWU5CLXhhdVVmZTQtVVJNSlJVN3VlYjU5N0kxRlhPMG9FTXQ4ZDdpMUJXVjJZUmtqeDZkT1pUb0ptRU9MM19ibFJ1OVlMeTRjYmt1cVBqRFRYd0F2aENmTmIzV1NpNl9HNm9ia1QtLTZSaE1ib2puWmFQcWc4NVU0NHQ2OWdSeWdlVFJpU084WlozYmNoVDZZWlZ4YUtIelR6bFVRWnBaYkxGWE5CMnpWcmFaTXZB?oc=5</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>30</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lynx penis enlarger sleeve: a realistic guide for men exploring non-invasive options - Portal CNJ</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 01:08:45 GMT</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNbWlSN3hkZEZQRHVMV2NwOHRBWVNtQkY3MzZYcTFEQ1FqN0x5SWhkWnJ2MEdPNTJkMGFtLUlJTEZFWFl2OFEzQkJVRlpNX0oyY2ltVDVmZnhneGw0TlI1OUZ3SDlEbV9VdUd6WlpLVS1CbWFUNlpwM01ZalQyU1FyejlkakJ0R01JREJnZEtxaXd6dG9nQ212WGFLM2xLYWhMVlFhdjVGWjNUajZZZHVEanhBbnVtclcwTW4zLVNrWUpSWkFLUTI1M1Zuel9SeUMyU0VPMG55bzY3YzNQdHJnWHRSR2JfMWRIcm1yamxaelBOMDduZjZ5N0JtWURVVlBfbU5DbUJhYk1Ba1Ny?oc=5</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>30</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Study reveals how menopause causes brain fog - fox5sandiego.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Tue, 21 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNMjdOdHlYQ28zLUtISU9kQ0l3QWQtZ1VnTFd3TG1ubEFBUWNGeU15RTA0SzQ0X05XUE94eXBhLVVuS0ZwdlJUMWpkZ0FHdU02aFB6N0hxLWZtdXpKUHg2NXJ1MFBjbEw1UlAtVVJQZ1JOdkwxR3JyV3VrLXkyaGdzaEhmZXFYQUFzbHBQOXZMcWRzTFhVUjgzR21xbVZkLW9j0gGmAUFVX3lxTE1sMFVmWHNNVjZwdFk3dXp2b2R3YkpfV3RFUnNySW14bkIwa1RLSmtEYkUxTjl4aVRRQS0wdnllNmNfMjliblE2TDhDRHdXdF9qYXpiSHl2QXRqc2F6WG5GV2tDNHRXeTJTQXBaUm4td294WlZqYWNJRzJhT1FuaURUNFpBamg5azk0Ri1NTVZUZENxWFd6N1JQLUJTaFZ0anVESWc2b3c?oc=5</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>30</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ransomware_Healthcare</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>(ransomware OR "cyber attack" OR "data breach") AND (hospital OR healthcare OR "medical centre" OR clinic OR pharmacy OR "health service" OR "patient data" OR "electronic health") AND (attacked OR disrupted OR encrypted OR offline OR incident OR breach OR warning)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Comparitech assesses healthcare ransomware decline in volume but escalates in impact, marking strategic shift - Industrial Cyber</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Thu, 30 Apr 2026 13:11:52 GMT</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxPbzN5MzM1c0kwTlJNTkw3WkNjN18tOXl4aDhZaVpLckVtQVhoNHU4R2E4MEtrZWdLUEg4aV83aDBYVGk3ZUdHNE1zSmN6V3NNd1lfSlhlaF9JY2t2aE1lVTNPdkh1QTVzWlFhU0g2c3ZjSXVIbk5SaVdsMm0zVV9EVkxoS1NKeDJUdng4ZllCTWYweG9tU1pWbE9kdHppdWFGOV9BVTRhNnNyMGoyYnZTcjRDMlFTR2NVcnJaM1BmXzBrMW8wZDd3bEpmZEpGNWl5Y0pnSVk4a3hhYUx5aVBnWA?oc=5</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>30</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ransomware_Incidents_UK_EU</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>(ransomware OR "cyber attack" OR "data breach") AND (NHS OR "local council" OR "local authority" OR "public sector" OR university OR school OR manufacturer OR retailer OR "law firm") AND (UK OR Britain OR England OR Scotland OR Wales OR Ireland OR Germany OR France OR Italy OR Spain OR Europe)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>International cyber attack disrupts swathe of universities and schools - BBC</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 01:17:55 GMT</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFAxZW9KSEdtMm1maTdXV181LVdFTWhUUElaMWhrd19KTUpTdW5wVXRBNmlPbXl6QkgwRjJlcW5HMFFLR01ZRTBXOXBCdml3UXpzMVNyQ09tcGlyUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>30</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FBI and Justice Department try to rebuild after wave of resignations and firings - PBS</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sun, 19 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNR2JmM0l6WUhiUlNkaW1VYVFDYkdfT2FZUG1rSnd2S3JacG5ldE9VcTd0S0pkby1xenRHSERldlNxc1AwSDRkNEhrQlpkZk52MVRfRFZEa1VKWFlSM29mSGFzQ3Z4alR0ZUFCVFhVOVZ3bXZicnZ2YzF6LS1aYXRuNXl3WF9YMlZ4N05XcnRrSWpiRGRtS2V5R25VVjlhQnBQcUh5dmw0akFYVW5yd19EdGxyWlUxQ0E?oc=5</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>30</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FBI Dallas Brings Awareness to Transnational Repression, Urges Public to Report Incidents to Law Enforcement - fbi.gov</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mon, 13 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQczRLV2ViNEJxWHlLb2tCVFNsS1JMNE01NFpWU2NteXdra290b0J1YUIxbVQ2QUJjOTMxM09TME8td1E2RlF6NlU3dWVoOGZ0NjNGNXZVdVZHaTdkdkRUV0toc29aVTlER2NZOEhYNEw3UWlqXzNoSlZKdGlhZGxuVFNOaDFKcDBvY2lQT29qcXFEUlRWbXB3U0xpeS1JV0hYRTFkYnA4TzFwQmN6YnlwdjBnMXdkRmpRbE9jZUk4XzlYSEFud19TMDhMemEzSVZIWmlHNVc4a3ktTS1sLWhvSlhjcmtRY3NpbnB3SG5PTGVFUW9XQU1Z?oc=5</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>30</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FBI seeks public’s help after a truck driver was possibly hijacked in Brevard County - WKMG</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Sun, 26 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOdy1lX1JJd1Jra2NsSjA2RnVNUzYwV1kya01kQTQtTnAteHpPeEF3aXZzWXRyNUpyQlFaVGtWZTAwWlJ5OEZTNUZmWDBpNVlfWmxmVFF3NEFaSUVWd3JCd2RzSGVmcWctVXR5ak9teE9FR3NxWnlMMkNLbk5HZWMxWTNBcE5RSkZhdjdGQi1mWGV2M0JOWVlkdElXMlUzSGZUVkdRRW5QRW5sWWJRVWU4d3h3SnphbjMwY3ZWZlhFWlNkSXA3cUZjVVlnbw?oc=5</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>30</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Bongino says he planted fake details to catch ‘snakes’ in FBI - The Hill</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Tue, 28 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNbzhZd2pXRmtlMFAwYUk2eFRVYXRVd3IzaG5vRFIyeEpKb3pTd2ZtS1p1Q2VUYXIzUE5OR1RSNjBXTVFmRHJtbHVSWmVZMGZLU1pBMkQ2RXFJT3YxZFJMWTNHTVVwYjZzd2lkWEx4YjA2aTRYaVpwTnJLbEFIbVlCRzVqVlU3Z9IBiwFBVV95cUxQM2JHT1FScUVFUlY2cmowcWlVY1ZmdlBQYVZIMnplZVNZVi1jWkFveUJMbmRobk4teS12Z292Q1MzS29MSEV1UjlwRWY0RzFzcWNOQmxIU1R4c1FoMk5wcFJCRm5sNkg4YTJjYlpTMjljOU1WeXo2enl5STljNW5OYndpUHBpcHNqV3RZ?oc=5</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>30</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Nancy Guthrie abduction: FBI analyzing DNA recovered from her home, sources say - ABC7 Los Angeles</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Thu, 16 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQVzEwM2VrMHdsWFM0TkVaSlNGdFlNa3pYNm1SdWhXWWJuc0M0QVY4cnYzOWJuZmM3NWoxWEc3Y1M3M1FBSTJjdF81bDQ0dzJTTF9QVWxTR0hoQW95NHlwUE5tN3dtUEJYM2hVWHFISDQ2V3BPNEFheExwcllwbTJ4cUJLd19ZY3hrdkZOamp2TUNWTkY5RlkyZ1VMU3Qtek9MTlE?oc=5</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>30</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ransomware_Tactics_Threats</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Singapore boffins get diverse SIEMs singing in harmony with agentic rule translation - The Register</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Tue, 05 May 2026 02:12:16 GMT</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPcGNlenZ0WnR2NXZfajFFQnFQVDRmU0N6d0Z2bnk0VXlNM3ltOXRjT09ES3Y5NXBIYmtpTUpMcGpvMWJRVWhyenNGRi15dGctUDhYRl9hVXN6Ul9TUnAyZXYwUkRzcXpsbjNqOWxiWDhVczB6ZWVlNlVSQTVTT2tzcXdqTnVyYVF5SVViXzNUWlNlcGZFd3VQR21ZZzRHMTJoNm9PN0djaWhudk5KX0M0?oc=5</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>30</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ransomware_Tactics_Threats</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Manufacturing absorbs 56% ransomware surge of global attacks in 2025, as RaaS, legacy OT, supply chains fuel spike - Industrial Cyber</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wed, 15 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOc1N4cXR2MGtmYVZrNFhuZ3AweHlBdUVwRG5CajB2UjVHRUs0bEROUGFnd21Rby11elFEVHZGTzZteDFjLWJ0THNRakNoTFJCM21ibXBQeG9OUnNWMkllbU9ieU05OG95ZGFyWC1uNnlxQlZ2RDdPVEZKRkN5S0ZFNjRLQ0E0Y1VobFdrSFVxOGQ4MW1ycWJzbzF5S2pkdmpEcjlPNl9ERlJiaU84MzJnWUxzbjE1b3hPa09kblRkTDhvVEo5emU1S2RGSmFadldldTNOODVhSXlWVkw0M1BCVG5IazViRnc?oc=5</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>30</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Critical Buffer Overflow Vulnerability in PAN-OS Exploited in-the-Wild - wiz.io</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 12:33:26 GMT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQOThjQzR2cXh2bVRWcEcwcHA2YWZGTTczUjc1dmlKQWtsRjVzZzRLRjJ1N2hzS2twbDhiejNhNDJlVi00UEZjSWZPcjZBRUZURGttMmgzemVVWExFUmY1OEJVQVB6RG52dWRiTkl5TkFZbFJZamxZOXVtYTc5M0VPNzhsbmhSVWF1UElPa2tUME42UHBfUFlR?oc=5</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>30</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ivanti customers confront yet another actively exploited zero-day - CyberScoop</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 21:59:16 GMT</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5hajI0N3NVXzBmY3hHZzBjV21GaUZ4TC1vdy1jekNQdnVZbjV2VFJtRHM4Q0VzRUh1Wlg0ek40S2NNbkY0VXFabVktWFdiaklPZmFqT2czbmJBaVVsV3JRZXZWZVNmamVhMkNHellRbC1KdkxVVGJZ?oc=5</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Critical 9.8 Weaver E-cology vulnerability actively exploited | news | SC Media - SC Media</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Tue, 05 May 2026 19:29:59 GMT</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPWThjdURva1RSdFBmUXlSaDg2ODJtRW1oLWpYbE9qNE0zOHY4SXhVRnk5eERna3RMVFdBSFRlR3FtN3NHaFZ1aDhsM1E5bzFtQTc5ck5xLWg5VGlQelFyTU16OVlFNzFqbVoyeTVFdDdaTFFwcTd0dlNfTjdSRm8zYkJLU0FaRi10bVJqQks5dTNNc1U?oc=5</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>30</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>New Ivanti EPMM 0-Day Vulnerability Actively Exploited in Attacks - CyberSecurityNews</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Thu, 07 May 2026 16:32:43 GMT</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE9OM0hHOTdSNndYR1JqUkhvVTNKOVpLY2dRNDJwTkRIM0NvSkdZMDJPcmNuZXVJY2JfbUZvUS1JaWlRZG9ZbnFNVFprWnBROWl1MDhGUGNpZWw4bDlGVDdfUW9feWMtTEc4VEHSAW9BVV95cUxOV01yMS1GY0h4eVVqTXpwRlZKZk0yTWRlSmxsNmt6akdpMGx5UG9MZzhoYW41TGQyZU1aOWFTdHc5UjdvT0pfMW1pNVBrQU52cHFIRUI5ZXY0Y0RzcWNSX0J6YXptOFNxdHplbmpxMEU?oc=5</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ransomware scum, other crims exploit 4 old Microsoft bugs - The Register</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Mon, 13 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOTXg0LUFXZDF6MVptVFlOWW53X09FUnNpamtiNDhuTkgxc0hmMTVNcFpOLWNIekl5R0x4RThZSzI1ZVJtZndnUVJOc3Q3ckx4NGVKajFTVUxuamFEbzlGU2xuZGROLXNscVJOTWNNYV9wM0Yyekg4cHVNUHpZQl94NWh1TQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>30</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Recent Apache ActiveMQ Vulnerability Exploited in the Wild - SecurityWeek</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Fri, 17 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQZ1lBa192TTVxQlk1OWFTSjk2ZExtYnh4QkVBTWZDYUl6N2RaUFN5aGdQR25ZQzg2VnZRSzhYaTR6NUZPa3c3enR3WmN4MERIOHhpa2pFX2phQUxDc0x1cktNcXVLalJ5YWRqR0x5NUZwUHRqbE1yR2o3a1lfd2ZjLTFZMVFPNlJxOWZhSWY4QWtzUdIBlwFBVV95cUxOaDNLZkkxcWQwdXNZVC0zcmhPLUVjZ2ktanlfMnVoS3l0UFRSN1pXU2hUZGRWV3pPQTlEMmZPeWFPaHJZeWlzMUVqS1RkUzctYkxDcnE3UWRuMk5qWmoxOXBzSUhvZ21rYlQ0Ynd1ZTN0bllmZjhfRnAxNEtVTW1kc1BhYzJfbEtwZVNWQThtd3VreE5vZDlv?oc=5</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>30</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Simply opening a PDF could trigger this Adobe Reader zero-day - Malwarebytes</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mon, 13 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNUW5CNlVaV2M1SFZ3RUN6bnRfelFnejJmV1NValMxdGE3RjNNUldFclZOcl9FeTRobTZKRWRiNklaTzhwWksxeXdJZF9JOTZ4M2tRTWVPSUFiWUtNSUhCck43aGMxeWZmb0x4NkRuQ2ZiNXRiLTgwZmRscEdFd0RCZ0l3Z2xNcm4xcHJ1STZ0RDlWeWRYbGhJc1dTd29QX3N5YUJ6bWxKTFgzdmpM?oc=5</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>30</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CISA Adds Actively Exploited Linux Root Access Bug CVE-2026-31431 to KEV - The Hacker News</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Sun, 03 May 2026 06:26:00 GMT</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNWGM1OVM2YXpMNEtXb3gtTzgzd1N5c0Z0NXk1VGNaU2dYbm9PemRxbkoxMTUxekdqczRDMXFSVTJKLXJQSU0zT2VLa1VtbXdFWmJ0THdibWNLTXdzQ3FaUVlNbjdfNGppYV9DU1NMRzJtM1dVTlJPb3FHTV9iUTFYNkpKTlo?oc=5</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>30</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A critical Palo Alto PAN-OS zero-day is being exploited in the wild - CyberScoop</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Wed, 06 May 2026 19:50:39 GMT</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQYVdGSDdxYnVzc0t2Uk5SUDJsVUlDNVgxQlVNdzI5SkluYWhBSlVPeDNkN2RTS1JCYm1Kd1dfTVdyazNCNl9WNVNEa2JJWjJlR1FSU1Buei1Yd0hWdHRrZ2U2VHZDMmpBWVdVaTh5WXRPTnphTUtDTzlLUnJrMzR0dWFLc2p4TUhNSlBRV3ROcU94OVZSeWc?oc=5</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>30</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Hackers exploit Marimo flaw to deploy NKAbuse malware from Hugging Face - BleepingComputer</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Thu, 16 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQU2duZUU0eVFWT1c1TzEtU2VRWUVhbnJHUWtuVFUtanFVb3c1UEhNZDNOTEhBbVBzOUZyYmx0LVI5bWhqMWdCQWU1blhON3ZDNEgyVUVodFpDQ19uZnc1MW9DQklRZXJnU1J0cFU4eXFRcUpjZWUxUXZFVFg5akNLUzk1S3BzSU5ZX1JKUDRKSlppWWhjUkZCQjhhclpRbno4N2d3N0doaXV6clgtS0tPYnhwdTd4NzBDTXlJ0gHAAUFVX3lxTE5xYW9QaGpOcU1aQURSa1c3OV8xSG5YcVVtWWFBWkZDQWhCc0IyWTF5OENsYm9wSlBxTEVmWV9GZVMwWkhaVHM5amVuTGhYOTNRSmYwdjFTYkd0TjFGVFdBaWVUWlRUNWZEc2xhdjQyaDlpOFg1UUJDODFRTldMaTFFSGRFV3hybDlScWdSUVVCTlhuOTRZeEdSRGY5Rk1BVTFSYzlZUjNGRTNnZFlQbDZoNUc5d01qcEIxenEzRDlTdg?oc=5</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Adobe issues emergency fix for Acrobat Reader flaw exploited in the wild (CVE-2026-34621) - Help Net Security</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Mon, 13 Apr 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNalBYODZnMlJFT3RGdzBwX0d5RzFIVng5NzJrQkNmdnlMYjNkaXgwS1BVblVjN0lEZzZTUFF4RVhiS3pTcjZXMGtUMmRMRzk4bW0tTWJDZ0dycjhWM0ZXR25zd2dRQzlFOUUxN3pfczkzbWJrR09idHZsRGFYSUhaQm02X1ZsbTZXc2U5RkN3c1otekpxc2t0RA?oc=5</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>30</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-13 08:38 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Darktrace Commentary on Canvas Ransomware Attack - iTWire</t>
+          <t>Foxconn Ransomware Attack Shows Nothing Is Safe Forever - WIRED</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 06:21:40 GMT</t>
+          <t>Tue, 12 May 2026 21:52:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNdThQNjJhS0tmYXNNVC03dGxsN3FsbkpvdTB1V3BjT1gzYlNveTAzYW1uYVRFUGpQdGhnVTlfLWhwd0ZpckpRNGN4X21LZ3dmSTZQamZ3Y0laS2pVWDM4bWxoLUR0ejNwYXRfNllMWlFSTDF6Q1FQd2tRVkNTTGZaX0prM0haQzdQYzdtbkg2aFNxcnlPWDJzUFRGWFg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQeUpEZnZQS2ZtWGFqa1I1Z0hoR0I0YUdHZXZsZFR5c2ZUM3ZZN3JJSkJIZmxwdGs0anNxMHE1Y3RlbDZONkRZd2o4S3RlZmNOWmkxREQ0OVVBekJuMURQbHRUQjVPaklXY0RrMU9admZrRHh0M2NXamFuZmlUWWhQYW52ZEM0cm14V3pXcA?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,27 +491,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Neurologist Shares Simple Ways to Keep the Brain Healthy - TODAY.com</t>
+          <t>Canvas hack: Company pays criminals to delete students' stolen data - BBC</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 15:14:05 GMT</t>
+          <t>Tue, 12 May 2026 10:31:23 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPaDRSZzNKTC0ycENBRm1XSnNBc1hGOTlaMFNnNTJLNDY0RmV3WmQzMXhsTW5SUzFhUHVIV3d5MVNCSVg1RUJGS05GWlFzRXVFbnYwTVBUaWZyOXo1SXNQbElfTWhVbHJWdkM0bFhTVWIzU09yV3lWN2IxazRaS0VDam8za28wQ0lvMkpWcHpodUZOckxvTGlPSlJKbkZqYWtsNU82cEF3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1BajhBQ1hESkkzSktfUHBjemFrMkhjaHJidVdGckM2YUJUMUtBODBmSzJMWTZJWHlMSFNSNENvQzJINWxNbEdKRkk5TTFfZ3pINUZSNlpJUGpHQQ?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -526,27 +526,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UAE weather: Chance of fog; temperature to reach 37°C in Abu Dhabi, Dubai - Khaleej Times</t>
+          <t>Ransomware sector reconsolidating as Qilin, LockBit, and The Gentlemen expand influence in Q1 2026 - Industrial Cyber</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 14:33:10 GMT</t>
+          <t>Tue, 12 May 2026 14:02:06 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE16U0pfanhIdU84dGxMMmpMYmx4T1M0cGVLUUVjX3NOZ3JMRjRkVGpDWWxxdlNUODFYQ2YwWDN1ZVpTVE14VHdVOG1jZzVHVjFMam1WQXlCUVRqNTh2MXBqeHJn0gFqQVVfeXFMTm40WkxMeUFyMFlCOUxVaGlmZnc0S25yZndtWWI2UnJfcnFpYU93c0xleEJ0WGNTbFNUaGtaRVhieTl2S2I5Mnk2aE1lbGY3d3BGWnYwaUFMMTRaS09SVnc3bjJSOUplUGpiZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPeFF0V1ktVzF5RzFqY09XdGxGYTVoX0VZeVlzM1dCQklPamxneUx0THpIUnItQjljR1VZR2dyRl9GNVVWNXFuNlVmNUNKYTQ2RWtIRnVYR0dHT2pwakREMkxhenNSR05RNUpmRTB2dERES2toNzRTQngzVFBJNHNsRzN1ak1fS254d2VKZ2ZjS3F2Y3MxOUNlTWg1YnZkdUpZWWNWbU9MOHcyaEpPWWltdjRyWnc3MEZTNlIxSjFZS3FlazBzVHp1Z1hmaGR3RG9p?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Tactics_Threats</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Google spotted an AI-developed zero-day before attackers could use it - CyberScoop</t>
+          <t>West Pharmaceutical warns of ransomware attack impacting business operations - The Record from Recorded Future News</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 13:01:25 GMT</t>
+          <t>Tue, 12 May 2026 19:13:07 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQaDVzZm1PdzJfMzBDV0JmT3NxQVFPeFkwNHdBTW1EUDJqS2FwMlpha0xSOTItOW9WblVQektWZHZjRDg5Q2NQQlZEaUMzUFlIMU1Pc0l6V21Sa2N2aFpERklBNVA3YVN6QzVXWkZCa1QyVEhxXzJfbHFtUk5Ib3ZFbzVGczBZZEpjT24tWU42bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxORG9yc3A0TDh2R2d4c29fbG9ZeC01WXlwakFSd0FzNmpvZUFBaUU0bVU0WXNvbEdvaWtZOGdLLVZlTllBczNKdHZhZ3l5M2dnVGZ2SlRSV1c1N0g0WWFSVlJmWm9PVnNEUU9JV1lxcEFTdU04bmpERzYzZUk0QW1CSXFXZVFUYU51TlY0VWZkSGJGMzRYUnc?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -596,33 +596,138 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ransomware_Vulnerabilities</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Google catches “first AI-assisted zero-day” as well as autonomous Android malware - Cybernews</t>
+          <t>Canvas hacked: After Canvas Instructure cyberattack ransomware agreement reached, personal information could still be at risk - ABC7 Chicago</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 16:37:22 GMT</t>
+          <t>Wed, 13 May 2026 00:41:54 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBtSEoyVGVWcGZRYTRENFNkTjN4V0dpZFU1N0k1X2RuTnh4Yzl0UmRBbThOSEhpWDdRRFJORnI4UzV6VFNDa3RDa21ualFTYTJuRl9JZGpOV2VQbGRoOEZ1TEtmQ0ZSNTJUdDhFNnctYTNXVXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQ2c4NDFpak5zY0NqMHBuYzBJZkhxZUVQRHBkb1k1dXRfc2NnbVFjUXZSTzVkUjQ4ZkVaQ1E2U0lMTm5vcEV0VXNQVFJTYy1hXy1QbnJTN2psZUtIRWlIQVEwYXFGUVNzRW5NNEU4Q3BBeDloU2hNOXFmNWU2aVJLQlVTTUV0SzJlN2JZeERmdm9RMTkyNF9wUW40Wi14U0diRVB1eHlaZkRxQ3ExbXh5OWVOX3ViaF96aXRFLXNHN1hSM2dmQ2toYVViQnpSb2NXMFhN0gHYAUFVX3lxTE93a1pxYThiZjRNNE5ueEtBYVIycXJXczJJOXFpNENoWFlvSzdEckI5bkE5M1lnWmwycVFqSXpSMnhfeHFzSkJzVkVVMkU5cmx6SmExeXo2RjQwZkxiaHg4dFNSSWtyRTZVSVFieTVxUmlaWlh5WDZidm1kdDFSTXU4ZVp3Z3o4dDJkNFF3UjJtSklWWnVWZTlaOFVlNGE4TUFlTlMxZklBYzJvdU9jLVI0ZHVWTlBGX1VZZXl6aWJ0OTh1SjVrOXNVU0ZDdjlTd2ZPU3g3dVFvMg?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ransomware_Activity</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>School Learning Company Reaches Deal with Hackers in Ransomware Attack - Newsradio WFLA Orlando</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 13:33:00 GMT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPbVZ0V0QtS3ExRF9mUkJXTHRmRTJ6NkdhaU92dkVWR2FtVW9Jam9SUzZKdFc3bDlraG4tT1oxLVJWUk1HS1RYQ2owazZ3ZFBmbkRCbEJMTEtTMTVMZ3AyM1Bsd1ZCUWZoa2V2NGFvQ1Jtb3MwSWZMcWR0RXFTeFF1eU9xdkhlVnNGM1NfajQ5VGZIeVo3Y1d5VjhseF9wNnRlcWNwYXZnS2kwd2lJeDhmRlVDblhTd1hrZ0tPOTBJUGhjOHFJMXk4OVBtc1ZhVjNYRnE0dEZkakVUQzQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cactus Announces Board and Executive Leadership Transitions - Stock Titan</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 21:15:00 GMT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWm9YVk50QnNzS2JlcFRheTBQaENQOWpGSmtlTW92VmtCZ0hqdW1BM2JjYmx1NEVxYUhlSFprTlRFYS10dWVGM1J1c1h1aFY0T1Q2UUtTZkFqMHF3N2xtMXN3M3lhUm0tOHE1dXp6QURUT05FNVFHMHlRWEExLTRwT2hxVjVKZmJPQjZxd3lhM3VCVURCLWNXdGdxTk9laEtfX2Fn?oc=5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Self-driving cars struggle to see at night or in fog – but imitating the human brain can make them safe - Yahoo Autos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 09:47:28 GMT</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPb2pBcjhIU0Y3eHEzUVl5TEhsSXhPbUFzYTRlWjFFN1VxMmRmWnRIQlMyTWhWZEZfR3VMa1NWSk5lNU5vZ2FHYkdURHdFYWZmRk9TZ3h2VHo5eDFjSGlpNXVabk9CNlM3d0plNlFTTkFUd2lZSXM0azd4cWJlU3FGSzN4cXBJaWhQNm9DY3czWnZPM1pzS1p0Y2FwbHNJQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-13 11:07 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Canvas hack: Company pays criminals to delete students' stolen data - BBC</t>
+          <t>Ransomware sector reconsolidating as Qilin, LockBit, and The Gentlemen expand influence in Q1 2026 - Industrial Cyber</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 10:31:23 GMT</t>
+          <t>Tue, 12 May 2026 14:02:06 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1BajhBQ1hESkkzSktfUHBjemFrMkhjaHJidVdGckM2YUJUMUtBODBmSzJMWTZJWHlMSFNSNENvQzJINWxNbEdKRkk5TTFfZ3pINUZSNlpJUGpHQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPeFF0V1ktVzF5RzFqY09XdGxGYTVoX0VZeVlzM1dCQklPamxneUx0THpIUnItQjljR1VZR2dyRl9GNVVWNXFuNlVmNUNKYTQ2RWtIRnVYR0dHT2pwakREMkxhenNSR05RNUpmRTB2dERES2toNzRTQngzVFBJNHNsRzN1ak1fS254d2VKZ2ZjS3F2Y3MxOUNlTWg1YnZkdUpZWWNWbU9MOHcyaEpPWWltdjRyWnc3MEZTNlIxSjFZS3FlazBzVHp1Z1hmaGR3RG9p?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ransomware sector reconsolidating as Qilin, LockBit, and The Gentlemen expand influence in Q1 2026 - Industrial Cyber</t>
+          <t>West Pharmaceutical warns of ransomware attack impacting business operations - The Record from Recorded Future News</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 14:02:06 GMT</t>
+          <t>Tue, 12 May 2026 19:13:07 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPeFF0V1ktVzF5RzFqY09XdGxGYTVoX0VZeVlzM1dCQklPamxneUx0THpIUnItQjljR1VZR2dyRl9GNVVWNXFuNlVmNUNKYTQ2RWtIRnVYR0dHT2pwakREMkxhenNSR05RNUpmRTB2dERES2toNzRTQngzVFBJNHNsRzN1ak1fS254d2VKZ2ZjS3F2Y3MxOUNlTWg1YnZkdUpZWWNWbU9MOHcyaEpPWWltdjRyWnc3MEZTNlIxSjFZS3FlazBzVHp1Z1hmaGR3RG9p?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxORG9yc3A0TDh2R2d4c29fbG9ZeC01WXlwakFSd0FzNmpvZUFBaUU0bVU0WXNvbEdvaWtZOGdLLVZlTllBczNKdHZhZ3l5M2dnVGZ2SlRSV1c1N0g0WWFSVlJmWm9PVnNEUU9JV1lxcEFTdU04bmpERzYzZUk0QW1CSXFXZVFUYU51TlY0VWZkSGJGMzRYUnc?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -571,17 +571,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>West Pharmaceutical warns of ransomware attack impacting business operations - The Record from Recorded Future News</t>
+          <t>Canvas hacked: After Canvas Instructure cyberattack ransomware agreement reached, personal information could still be at risk - ABC7 Chicago</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 19:13:07 GMT</t>
+          <t>Wed, 13 May 2026 00:41:54 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxORG9yc3A0TDh2R2d4c29fbG9ZeC01WXlwakFSd0FzNmpvZUFBaUU0bVU0WXNvbEdvaWtZOGdLLVZlTllBczNKdHZhZ3l5M2dnVGZ2SlRSV1c1N0g0WWFSVlJmWm9PVnNEUU9JV1lxcEFTdU04bmpERzYzZUk0QW1CSXFXZVFUYU51TlY0VWZkSGJGMzRYUnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQ2c4NDFpak5zY0NqMHBuYzBJZkhxZUVQRHBkb1k1dXRfc2NnbVFjUXZSTzVkUjQ4ZkVaQ1E2U0lMTm5vcEV0VXNQVFJTYy1hXy1QbnJTN2psZUtIRWlIQVEwYXFGUVNzRW5NNEU4Q3BBeDloU2hNOXFmNWU2aVJLQlVTTUV0SzJlN2JZeERmdm9RMTkyNF9wUW40Wi14U0diRVB1eHlaZkRxQ3ExbXh5OWVOX3ViaF96aXRFLXNHN1hSM2dmQ2toYVViQnpSb2NXMFhN0gHYAUFVX3lxTE93a1pxYThiZjRNNE5ueEtBYVIycXJXczJJOXFpNENoWFlvSzdEckI5bkE5M1lnWmwycVFqSXpSMnhfeHFzSkJzVkVVMkU5cmx6SmExeXo2RjQwZkxiaHg4dFNSSWtyRTZVSVFieTVxUmlaWlh5WDZidm1kdDFSTXU4ZVp3Z3o4dDJkNFF3UjJtSklWWnVWZTlaOFVlNGE4TUFlTlMxZklBYzJvdU9jLVI0ZHVWTlBGX1VZZXl6aWJ0OTh1SjVrOXNVU0ZDdjlTd2ZPU3g3dVFvMg?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -606,17 +606,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Canvas hacked: After Canvas Instructure cyberattack ransomware agreement reached, personal information could still be at risk - ABC7 Chicago</t>
+          <t>School Learning Company Reaches Deal with Hackers in Ransomware Attack - 1290 WJNO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 00:41:54 GMT</t>
+          <t>Tue, 12 May 2026 13:33:00 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQ2c4NDFpak5zY0NqMHBuYzBJZkhxZUVQRHBkb1k1dXRfc2NnbVFjUXZSTzVkUjQ4ZkVaQ1E2U0lMTm5vcEV0VXNQVFJTYy1hXy1QbnJTN2psZUtIRWlIQVEwYXFGUVNzRW5NNEU4Q3BBeDloU2hNOXFmNWU2aVJLQlVTTUV0SzJlN2JZeERmdm9RMTkyNF9wUW40Wi14U0diRVB1eHlaZkRxQ3ExbXh5OWVOX3ViaF96aXRFLXNHN1hSM2dmQ2toYVViQnpSb2NXMFhN0gHYAUFVX3lxTE93a1pxYThiZjRNNE5ueEtBYVIycXJXczJJOXFpNENoWFlvSzdEckI5bkE5M1lnWmwycVFqSXpSMnhfeHFzSkJzVkVVMkU5cmx6SmExeXo2RjQwZkxiaHg4dFNSSWtyRTZVSVFieTVxUmlaWlh5WDZidm1kdDFSTXU4ZVp3Z3o4dDJkNFF3UjJtSklWWnVWZTlaOFVlNGE4TUFlTlMxZklBYzJvdU9jLVI0ZHVWTlBGX1VZZXl6aWJ0OTh1SjVrOXNVU0ZDdjlTd2ZPU3g3dVFvMg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTHF3OUhrNjhDNkNVeW1UVnhra1pZbGdOT0tCS2ZVZVZoRlpIU3h0Ul8wZXBjeHFPdVg2cnkzeEtyU1RKeG5TdzBtQ0RzSTAtaEd1dlFoTVByXzdPNnJKRUZWa0xZcGhRdXd2emtRbmZ1TUR5N1p0MU1FeERnOE5VcHVvbTZKQUxDTExlQ0xwNDd6TFZ1ME5qbEhfM0psdG1ueUtNY3hlUFM5NVpPb3NKeVVLRnJvTDhQakp1T0swWHZTNHVtUjdhT2ZEdURFeGZQMXc?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -631,103 +631,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>School Learning Company Reaches Deal with Hackers in Ransomware Attack - Newsradio WFLA Orlando</t>
+          <t>Cactus Announces Board and Executive Leadership Transitions - Stock Titan</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 13:33:00 GMT</t>
+          <t>Tue, 12 May 2026 21:15:00 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPbVZ0V0QtS3ExRF9mUkJXTHRmRTJ6NkdhaU92dkVWR2FtVW9Jam9SUzZKdFc3bDlraG4tT1oxLVJWUk1HS1RYQ2owazZ3ZFBmbkRCbEJMTEtTMTVMZ3AyM1Bsd1ZCUWZoa2V2NGFvQ1Jtb3MwSWZMcWR0RXFTeFF1eU9xdkhlVnNGM1NfajQ5VGZIeVo3Y1d5VjhseF9wNnRlcWNwYXZnS2kwd2lJeDhmRlVDblhTd1hrZ0tPOTBJUGhjOHFJMXk4OVBtc1ZhVjNYRnE0dEZkakVUQzQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWm9YVk50QnNzS2JlcFRheTBQaENQOWpGSmtlTW92VmtCZ0hqdW1BM2JjYmx1NEVxYUhlSFprTlRFYS10dWVGM1J1c1h1aFY0T1Q2UUtTZkFqMHF3N2xtMXN3M3lhUm0tOHE1dXp6QURUT05FNVFHMHlRWEExLTRwT2hxVjVKZmJPQjZxd3lhM3VCVURCLWNXdGdxTk9laEtfX2Fn?oc=5</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ransomware_Groups_New</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Cactus Announces Board and Executive Leadership Transitions - Stock Titan</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Tue, 12 May 2026 21:15:00 GMT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWm9YVk50QnNzS2JlcFRheTBQaENQOWpGSmtlTW92VmtCZ0hqdW1BM2JjYmx1NEVxYUhlSFprTlRFYS10dWVGM1J1c1h1aFY0T1Q2UUtTZkFqMHF3N2xtMXN3M3lhUm0tOHE1dXp6QURUT05FNVFHMHlRWEExLTRwT2hxVjVKZmJPQjZxd3lhM3VCVURCLWNXdGdxTk9laEtfX2Fn?oc=5</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Ransomware_Groups_New</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Self-driving cars struggle to see at night or in fog – but imitating the human brain can make them safe - Yahoo Autos</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Tue, 12 May 2026 09:47:28 GMT</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPb2pBcjhIU0Y3eHEzUVl5TEhsSXhPbUFzYTRlWjFFN1VxMmRmWnRIQlMyTWhWZEZfR3VMa1NWSk5lNU5vZ2FHYkdURHdFYWZmRk9TZ3h2VHo5eDFjSGlpNXVabk9CNlM3d0plNlFTTkFUd2lZSXM0azd4cWJlU3FGSzN4cXBJaWhQNm9DY3czWnZPM1pzS1p0Y2FwbHNJQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-14 08:31 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Foxconn Ransomware Attack Shows Nothing Is Safe Forever - WIRED</t>
+          <t>Canvas Owner Reaches Agreement With Cybercriminals After Ransomware Attack - Infosecurity Magazine</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 21:52:00 GMT</t>
+          <t>Wed, 13 May 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQeUpEZnZQS2ZtWGFqa1I1Z0hoR0I0YUdHZXZsZFR5c2ZUM3ZZN3JJSkJIZmxwdGs0anNxMHE1Y3RlbDZONkRZd2o4S3RlZmNOWmkxREQ0OVVBekJuMURQbHRUQjVPaklXY0RrMU9admZrRHh0M2NXamFuZmlUWWhQYW52ZEM0cm14V3pXcA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaGUyNnZ0TzBrNmQwSVhreE9OeVdTcjQtbTlnYnZfcExfcWp0TWIzeGo2RU9GVXVHZVQ4WDM5SDZ2VUp6TkpWb0JBdnlTV1kzYXNiX0xGYS0yOXpCV0VnNGVCbkRxU2s5UWVmQlczZi1iVDRhS1ZTbnlza3pPMkVuVg?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ransomware sector reconsolidating as Qilin, LockBit, and The Gentlemen expand influence in Q1 2026 - Industrial Cyber</t>
+          <t>Apple Supplier Foxconn Hit With Ransomware Attack - PYMNTS.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 14:02:06 GMT</t>
+          <t>Wed, 13 May 2026 15:53:52 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPeFF0V1ktVzF5RzFqY09XdGxGYTVoX0VZeVlzM1dCQklPamxneUx0THpIUnItQjljR1VZR2dyRl9GNVVWNXFuNlVmNUNKYTQ2RWtIRnVYR0dHT2pwakREMkxhenNSR05RNUpmRTB2dERES2toNzRTQngzVFBJNHNsRzN1ak1fS254d2VKZ2ZjS3F2Y3MxOUNlTWg1YnZkdUpZWWNWbU9MOHcyaEpPWWltdjRyWnc3MEZTNlIxSjFZS3FlazBzVHp1Z1hmaGR3RG9p?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNaXFPc2VLY1NBaENsN1hBTkFpdW94UFFLak1rWk01R2pubW93RF9GeTBYZ3ZYX1hyNWVmVXZBMjAtdjBJaE5aSmRWbkJEZFo3TmpnaVBXSXh3UTdhM24walJYZDRaWUJfeHZpc3J2SFh2ZXdqdmFjWVRacnJ2MEgyNmZ4amloUWprSjF1VVhydEpSWWQ3TDJ5d3RFRzNWTUJVbV9Z?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>West Pharmaceutical warns of ransomware attack impacting business operations - The Record from Recorded Future News</t>
+          <t>After Nevada's ransomware attack, security upgrades have been 'game-changing,' says state CIO - StateScoop</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 19:13:07 GMT</t>
+          <t>Wed, 13 May 2026 18:18:13 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxORG9yc3A0TDh2R2d4c29fbG9ZeC01WXlwakFSd0FzNmpvZUFBaUU0bVU0WXNvbEdvaWtZOGdLLVZlTllBczNKdHZhZ3l5M2dnVGZ2SlRSV1c1N0g0WWFSVlJmWm9PVnNEUU9JV1lxcEFTdU04bmpERzYzZUk0QW1CSXFXZVFUYU51TlY0VWZkSGJGMzRYUnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPNktkbS1vNkw0MEQxbkR6UXdPbkdsUXBMMmRwOHg3ajAtRmYtbkxhQm1FMm9XQkxicWtSbS1oc2pRUHNGSjN5Q2lsYkk4M0dvNndweU1sdTNnT3V4bFBkeXpHay1MWHM3UVB5M0c3QmJvb0ZfVlhhM01kZkFaM1hHY3JIdnd6ZVE2NjVheU1NRVVMajFROG5RWWhqNGJoY1Nmem9XSXVYeHUyY1ZMLTdmMDBmdGVFTlY3Ymc?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,103 +561,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Tactics_Threats</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Canvas hacked: After Canvas Instructure cyberattack ransomware agreement reached, personal information could still be at risk - ABC7 Chicago</t>
+          <t>Pulling the Plug: Why Internet Shutdowns Fail as Cyber Defense - OODAloop</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 00:41:54 GMT</t>
+          <t>Wed, 13 May 2026 15:04:23 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQ2c4NDFpak5zY0NqMHBuYzBJZkhxZUVQRHBkb1k1dXRfc2NnbVFjUXZSTzVkUjQ4ZkVaQ1E2U0lMTm5vcEV0VXNQVFJTYy1hXy1QbnJTN2psZUtIRWlIQVEwYXFGUVNzRW5NNEU4Q3BBeDloU2hNOXFmNWU2aVJLQlVTTUV0SzJlN2JZeERmdm9RMTkyNF9wUW40Wi14U0diRVB1eHlaZkRxQ3ExbXh5OWVOX3ViaF96aXRFLXNHN1hSM2dmQ2toYVViQnpSb2NXMFhN0gHYAUFVX3lxTE93a1pxYThiZjRNNE5ueEtBYVIycXJXczJJOXFpNENoWFlvSzdEckI5bkE5M1lnWmwycVFqSXpSMnhfeHFzSkJzVkVVMkU5cmx6SmExeXo2RjQwZkxiaHg4dFNSSWtyRTZVSVFieTVxUmlaWlh5WDZidm1kdDFSTXU4ZVp3Z3o4dDJkNFF3UjJtSklWWnVWZTlaOFVlNGE4TUFlTlMxZklBYzJvdU9jLVI0ZHVWTlBGX1VZZXl6aWJ0OTh1SjVrOXNVU0ZDdjlTd2ZPU3g3dVFvMg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNQXpoMjZFeHZwTUhfUGdrbUhmSTRlbHFnV1VXMWpscGdUV3JsanRlNVFMWjktX0xwaHdBTWlZTlZCTTRCSERKbEVHVzg2Y0xXVmZ1MS1DTUI4UzFlN1dEWVVJMnZid2gzcFRnbnF6ajh1akV3RTZhbnZTTEp1dVJ0WmlhSG5QbjgyQldRaGhrRWxsTFo0WF9kRVk2SkdodzFCT1NwS2JyYlpDOU8tcUtpMENkZ2tuNWc?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ransomware_Activity</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>School Learning Company Reaches Deal with Hackers in Ransomware Attack - 1290 WJNO</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Tue, 12 May 2026 13:33:00 GMT</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTHF3OUhrNjhDNkNVeW1UVnhra1pZbGdOT0tCS2ZVZVZoRlpIU3h0Ul8wZXBjeHFPdVg2cnkzeEtyU1RKeG5TdzBtQ0RzSTAtaEd1dlFoTVByXzdPNnJKRUZWa0xZcGhRdXd2emtRbmZ1TUR5N1p0MU1FeERnOE5VcHVvbTZKQUxDTExlQ0xwNDd6TFZ1ME5qbEhfM0psdG1ueUtNY3hlUFM5NVpPb3NKeVVLRnJvTDhQakp1T0swWHZTNHVtUjdhT2ZEdURFeGZQMXc?oc=5</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ransomware_Groups_New</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Cactus Announces Board and Executive Leadership Transitions - Stock Titan</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Tue, 12 May 2026 21:15:00 GMT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOWm9YVk50QnNzS2JlcFRheTBQaENQOWpGSmtlTW92VmtCZ0hqdW1BM2JjYmx1NEVxYUhlSFprTlRFYS10dWVGM1J1c1h1aFY0T1Q2UUtTZkFqMHF3N2xtMXN3M3lhUm0tOHE1dXp6QURUT05FNVFHMHlRWEExLTRwT2hxVjVKZmJPQjZxd3lhM3VCVURCLWNXdGdxTk9laEtfX2Fn?oc=5</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-15 08:43 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Canvas Owner Reaches Agreement With Cybercriminals After Ransomware Attack - Infosecurity Magazine</t>
+          <t>News - Ransomware attack on American Lending Center compromised over 123K individuals - teiss</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 14:30:00 GMT</t>
+          <t>Thu, 14 May 2026 22:51:34 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNaGUyNnZ0TzBrNmQwSVhreE9OeVdTcjQtbTlnYnZfcExfcWp0TWIzeGo2RU9GVXVHZVQ4WDM5SDZ2VUp6TkpWb0JBdnlTV1kzYXNiX0xGYS0yOXpCV0VnNGVCbkRxU2s5UWVmQlczZi1iVDRhS1ZTbnlza3pPMkVuVg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxObnIwQkVHV3JkTk83UGVoZkF3Q1JzMzJ1TUxpS19OeDIxSlpaUEVJVmh4M3Z2bktVclVSckNkMGhyRllOa3d5UG1oRGhZQXNPNXd1aXJheGR5NkxDa2IyRUtSWXRZSHVFTmpDeEJpQmpPZEZfVF9JQVQ3enFNN19aV0dqOXc3Wnc4aUpYMmhwRkpWaG5ETjNWVE0zQktPX0FEeEFVOExvVk1MQ1l2dHRXVGlJQQ?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Apple Supplier Foxconn Hit With Ransomware Attack - PYMNTS.com</t>
+          <t>West Pharmaceutical starts restoring operations after ransomware attack - Cybersecurity Dive</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 15:53:52 GMT</t>
+          <t>Thu, 14 May 2026 15:23:43 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNaXFPc2VLY1NBaENsN1hBTkFpdW94UFFLak1rWk01R2pubW93RF9GeTBYZ3ZYX1hyNWVmVXZBMjAtdjBJaE5aSmRWbkJEZFo3TmpnaVBXSXh3UTdhM24walJYZDRaWUJfeHZpc3J2SFh2ZXdqdmFjWVRacnJ2MEgyNmZ4amloUWprSjF1VVhydEpSWWQ3TDJ5d3RFRzNWTUJVbV9Z?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOTkRPeVZ0NkZFVEZlVDhuWFFLRzlnTUtrTFM5cnI1ZnJlOFFVWVg5VDBCTHpmc1E1NlZNZnJCVjg0VWE0dWpqLWhVWnE4NEhPc196Wnp3TUFDa1k5a3puZkFjeldDVnctT2tacDRZRTNMVDc5UGY2TnlYcU1jRDRoU1kyNlcyQTFfRWo4aDFNdzZUbFBDbk40WVdZUTlGejFLR2UyaU5ma0U?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -536,17 +536,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>After Nevada's ransomware attack, security upgrades have been 'game-changing,' says state CIO - StateScoop</t>
+          <t>Foxconn factories resume operations after ransomware attack | brief | SC Media - SC Media</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 18:18:13 GMT</t>
+          <t>Thu, 14 May 2026 14:52:04 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPNktkbS1vNkw0MEQxbkR6UXdPbkdsUXBMMmRwOHg3ajAtRmYtbkxhQm1FMm9XQkxicWtSbS1oc2pRUHNGSjN5Q2lsYkk4M0dvNndweU1sdTNnT3V4bFBkeXpHay1MWHM3UVB5M0c3QmJvb0ZfVlhhM01kZkFaM1hHY3JIdnd6ZVE2NjVheU1NRVVMajFROG5RWWhqNGJoY1Nmem9XSXVYeHUyY1ZMLTdmMDBmdGVFTlY3Ymc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOOXExTTdCRFllY1MxZjlIcVlzRXRaZzFxMkpsQzdCMnUwc1pua05LMllCUzQzR3JFbW00LThKMzVXOW0yRTlobHZVaDJfTHhXTGdfU0p5ZS1ZNDBFX0ZkSW5RWlNOQy1oa2s4NDI1WWQ5RG93MVN6OFE4U21kcGM4c2Q3Uk1zZWxSNVZ6SjNIajUtZVE?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Tactics_Threats</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("double extortion" OR "triple extortion" OR "RaaS" OR "ransomware-as-a-service" OR "initial access broker" OR "zero day exploit" OR "credential theft" OR "MFA bypass" OR "new ransomware" OR "ransomware variant" OR "AI-powered ransomware" OR "OT ransomware" OR "ICS ransomware" OR "wiper malware" OR "supply chain attack") AND (ransomware OR malware OR "threat actor" OR technique OR emerging OR advisory OR warning OR discovered)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pulling the Plug: Why Internet Shutdowns Fail as Cyber Defense - OODAloop</t>
+          <t>Foxconn ransomware attack sees Apple and Nvidia data stolen - Notebookcheck</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 15:04:23 GMT</t>
+          <t>Thu, 14 May 2026 14:03:00 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNQXpoMjZFeHZwTUhfUGdrbUhmSTRlbHFnV1VXMWpscGdUV3JsanRlNVFMWjktX0xwaHdBTWlZTlZCTTRCSERKbEVHVzg2Y0xXVmZ1MS1DTUI4UzFlN1dEWVVJMnZid2gzcFRnbnF6ajh1akV3RTZhbnZTTEp1dVJ0WmlhSG5QbjgyQldRaGhrRWxsTFo0WF9kRVk2SkdodzFCT1NwS2JyYlpDOU8tcUtpMENkZ2tuNWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPb3hUQktuZ0E1UTFodGRkTVUtbEl6X3dRVFJ1U1ptYnlqR1VBN3R2d3VUVmtmWExPeXRKSk1uYUs0eGIyaDJaa0xSQ25leng5NEp6akFnaGpGQUxaRGNTWGpGS0JLRlJ0bFhmVkJNT3VNanc2bE9lY3IxWW54VThjYjYtaGJIeDlDOEc2SFlVWDRyR08xYUxMZ29UZ3VUZXR5Zy03OFV4Zw?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-16 07:54 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,27 +456,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Healthcare</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>(ransomware OR "cyber attack" OR "data breach") AND (hospital OR healthcare OR "medical centre" OR clinic OR pharmacy OR "health service" OR "patient data" OR "electronic health") AND (attacked OR disrupted OR encrypted OR offline OR incident OR breach OR warning)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>News - Ransomware attack on American Lending Center compromised over 123K individuals - teiss</t>
+          <t>Ransomware Groups Claim Responsibility for Attacks on 3 Healthcare Providers - The HIPAA Journal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thu, 14 May 2026 22:51:34 GMT</t>
+          <t>Fri, 15 May 2026 10:09:54 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxObnIwQkVHV3JkTk83UGVoZkF3Q1JzMzJ1TUxpS19OeDIxSlpaUEVJVmh4M3Z2bktVclVSckNkMGhyRllOa3d5UG1oRGhZQXNPNXd1aXJheGR5NkxDa2IyRUtSWXRZSHVFTmpDeEJpQmpPZEZfVF9JQVQ3enFNN19aV0dqOXc3Wnc4aUpYMmhwRkpWaG5ETjNWVE0zQktPX0FEeEFVOExvVk1MQ1l2dHRXVGlJQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWk5IVS1JR00ydTM4WlQ1VHB1eVJVSW1KejRub1RQVEoyWV9abmlhYjYzM0VmU2tKRTNKM2JFZ2pJeWpIemtzVWVKQ0Z0VXpPNGNjUmd3S0xFV0FsQk93RmxiMlI1OHN6YVpFcU1GMW4zRFdHVzd3QVlFQmFTZXI3YXVRdHdDOElRWlZWendPdlNkNWhWZnBtMzhiT3JfZWN0TU1BYURR?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,27 +491,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Response</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>West Pharmaceutical starts restoring operations after ransomware attack - Cybersecurity Dive</t>
+          <t>FBI offers $200K reward for former service member accused of espionage - NewsNation</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Thu, 14 May 2026 15:23:43 GMT</t>
+          <t>Fri, 15 May 2026 17:16:34 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOTkRPeVZ0NkZFVEZlVDhuWFFLRzlnTUtrTFM5cnI1ZnJlOFFVWVg5VDBCTHpmc1E1NlZNZnJCVjg0VWE0dWpqLWhVWnE4NEhPc196Wnp3TUFDa1k5a3puZkFjeldDVnctT2tacDRZRTNMVDc5UGY2TnlYcU1jRDRoU1kyNlcyQTFfRWo4aDFNdzZUbFBDbk40WVdZUTlGejFLR2UyaU5ma0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE54cFdlVzZMNU1rS0ROcG9lc21uN2VSRlBnMXdJSlIzLVhJQ1hnM2pvbFdfR2pnVjBqWHI4cFhEV3BVTnAwaXl6Q1h6S21Jdm9uZS15QTIwZFppYTQ3VEpxOWFiMHF1YU1rX0R2ZGFWbkFfWTJoVnfSAXtBVV95cUxNNWlibFNVM1dzc0p4T0xfS29jT3VJVTVCR3hLOW10NHNYUEV2RlJjQS1fVDNzVXd2SEh5SEZtZm42NDRqVXppbFUxb2tjTjRZVnAzcDc3OFFNM0tsWDczRHB3QnppRXlmbG0xeHF2RXJ6dG1YYkU1VnRVQ0E?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -526,68 +526,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Vulnerabilities</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Foxconn factories resume operations after ransomware attack | brief | SC Media - SC Media</t>
+          <t>Microsoft Warns of Exchange Server Zero-Day Exploited in the Wild - SecurityWeek</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thu, 14 May 2026 14:52:04 GMT</t>
+          <t>Fri, 15 May 2026 12:06:53 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOOXExTTdCRFllY1MxZjlIcVlzRXRaZzFxMkpsQzdCMnUwc1pua05LMllCUzQzR3JFbW00LThKMzVXOW0yRTlobHZVaDJfTHhXTGdfU0p5ZS1ZNDBFX0ZkSW5RWlNOQy1oa2s4NDI1WWQ5RG93MVN6OFE4U21kcGM4c2Q3Uk1zZWxSNVZ6SjNIajUtZVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQOU83eGxyOUdORWNCUzFxSmJWcENvWTdLeDRoTGRSdUhUWTNKTDR2cVNXOVpqazNLdGtjLTFrRXNTeXUyZ1dMZExWOWRONXgtYU5CN3RndlRYVzJMd3MyOG9MaWhLTzdqbFdNTFgtVzh5enQ1b0lyLXo0WUZWblhCaHQ5bXZoZ0N5RGtEUjY5UFlfazd2MjNEMmRZZ9IBoAFBVV95cUxOeTI0Z3lsV1NsY0c5b1V5YVlFUHBmMV9BcEM4RXdiejlJWV9WTHlDYkVXR1ZIQjBydkUzU3RqQi1PQ0I2bEJKMGQ0TXl0ZjlOS29tX1R1NDZkaEFpOE1ZTHRka2tKSWJoYUhfczQ4VzlUeEttUVpwTGNZX0lfU0RKZkVCZkRNTlRWSjB1WnpYRDFicVhNQldneDVGSFlZT2Ix?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ransomware_Activity</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Foxconn ransomware attack sees Apple and Nvidia data stolen - Notebookcheck</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Thu, 14 May 2026 14:03:00 GMT</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPb3hUQktuZ0E1UTFodGRkTVUtbEl6X3dRVFJ1U1ptYnlqR1VBN3R2d3VUVmtmWExPeXRKSk1uYUs0eGIyaDJaa0xSQ25leng5NEp6akFnaGpGQUxaRGNTWGpGS0JLRlJ0bFhmVkJNT3VNanc2bE9lY3IxWW54VThjYjYtaGJIeDlDOEc2SFlVWDRyR08xYUxMZ29UZ3VUZXR5Zy03OFV4Zw?oc=5</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-17 08:13 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,27 +456,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ransomware_Healthcare</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(ransomware OR "cyber attack" OR "data breach") AND (hospital OR healthcare OR "medical centre" OR clinic OR pharmacy OR "health service" OR "patient data" OR "electronic health") AND (attacked OR disrupted OR encrypted OR offline OR incident OR breach OR warning)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ransomware Groups Claim Responsibility for Attacks on 3 Healthcare Providers - The HIPAA Journal</t>
+          <t>Iran war: Finding steadiness in uncertain times - The Jerusalem Post</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Fri, 15 May 2026 10:09:54 GMT</t>
+          <t>Sat, 16 May 2026 19:41:53 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWk5IVS1JR00ydTM4WlQ1VHB1eVJVSW1KejRub1RQVEoyWV9abmlhYjYzM0VmU2tKRTNKM2JFZ2pJeWpIemtzVWVKQ0Z0VXpPNGNjUmd3S0xFV0FsQk93RmxiMlI1OHN6YVpFcU1GMW4zRFdHVzd3QVlFQmFTZXI3YXVRdHdDOElRWlZWendPdlNkNWhWZnBtMzhiT3JfZWN0TU1BYURR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE53YXVWeFdKeHhUbjBHVDdnS3RUX3BJeVZoSUozZmgwT3ZXQzJfdXNGMzZQU2V2X3NBQUd3b3NDUGdpbGQ3dlVTRVowR3FOR3FtZzV1b0FtOWp4OWFtTWhxNWpjR3RNeTRvOG85MVJIeTJBQXBFUDRXZ09iMjA?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,68 +491,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Response</t>
+          <t>Ransomware_Vulnerabilities</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FBI offers $200K reward for former service member accused of espionage - NewsNation</t>
+          <t>Critical Microsoft Exchange Server Vulnerability Actively Exploited in Attacks - CyberSecurityNews</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fri, 15 May 2026 17:16:34 GMT</t>
+          <t>Sat, 16 May 2026 10:08:55 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE54cFdlVzZMNU1rS0ROcG9lc21uN2VSRlBnMXdJSlIzLVhJQ1hnM2pvbFdfR2pnVjBqWHI4cFhEV3BVTnAwaXl6Q1h6S21Jdm9uZS15QTIwZFppYTQ3VEpxOWFiMHF1YU1rX0R2ZGFWbkFfWTJoVnfSAXtBVV95cUxNNWlibFNVM1dzc0p4T0xfS29jT3VJVTVCR3hLOW10NHNYUEV2RlJjQS1fVDNzVXd2SEh5SEZtZm42NDRqVXppbFUxb2tjTjRZVnAzcDc3OFFNM0tsWDczRHB3QnppRXlmbG0xeHF2RXJ6dG1YYkU1VnRVQ0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOVEVUb05Fbmd1dEdMU2RudVFoV0dHYmMzMS1IMVpFVlNJLUlwMkxOWHhHWEkzLUJtaTV5Vk0tYTFpT1JhU2ZkVXZpNERQNklkYWpLQ3NBLXozNUxuNXZCMTF5VDFHd3RwWjdkQzZFdGlxUzQxVS1yazYxR2hHSWxhWDhISC1tV0HSAYwBQVVfeXFMTjl3RTIxTmVYVGhKSVdEWVBNdHVWT1dFbkdwRkY3OXpNdm5xVC0tRjN1N1k4dWNkNkNneEJxZzlIbHpKamZnYUQ0cGVJaklJWHl1OFRGUzRQQ0tNLWIwdDVGbTFSdDE3WUtaQTJPR2VwQkNoanVTWUNuQnA0SGtKMU9sWVg1ZDk3M0VPb2Q?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ransomware_Vulnerabilities</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Microsoft Warns of Exchange Server Zero-Day Exploited in the Wild - SecurityWeek</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Fri, 15 May 2026 12:06:53 GMT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQOU83eGxyOUdORWNCUzFxSmJWcENvWTdLeDRoTGRSdUhUWTNKTDR2cVNXOVpqazNLdGtjLTFrRXNTeXUyZ1dMZExWOWRONXgtYU5CN3RndlRYVzJMd3MyOG9MaWhLTzdqbFdNTFgtVzh5enQ1b0lyLXo0WUZWblhCaHQ5bXZoZ0N5RGtEUjY5UFlfazd2MjNEMmRZZ9IBoAFBVV95cUxOeTI0Z3lsV1NsY0c5b1V5YVlFUHBmMV9BcEM4RXdiejlJWV9WTHlDYkVXR1ZIQjBydkUzU3RqQi1PQ0I2bEJKMGQ0TXl0ZjlOS29tX1R1NDZkaEFpOE1ZTHRka2tKSWJoYUhfczQ4VzlUeEttUVpwTGNZX0lfU0RKZkVCZkRNTlRWSjB1WnpYRDFicVhNQldneDVGSFlZT2Ix?oc=5</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-18 09:45 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,27 +456,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Iran war: Finding steadiness in uncertain times - The Jerusalem Post</t>
+          <t>Foxconn Suffers Ransomware Attack With Important Project Files From Apple Stolen - ilounge.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sat, 16 May 2026 19:41:53 GMT</t>
+          <t>Mon, 18 May 2026 04:51:36 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE53YXVWeFdKeHhUbjBHVDdnS3RUX3BJeVZoSUozZmgwT3ZXQzJfdXNGMzZQU2V2X3NBQUd3b3NDUGdpbGQ3dlVTRVowR3FOR3FtZzV1b0FtOWp4OWFtTWhxNWpjR3RNeTRvOG85MVJIeTJBQXBFUDRXZ09iMjA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPOG5DelA3dElSaTBEX3ZFV3JRcUV5N1FYbEJtbXpHallOOEVhNF9aXzFzWVhSMjRsM1lyVkZvMjhja3ZVZTBDTHJPTkM0TUg0UXJ3SlNHWFhHWVVRYXRqNnlKc0c1bkxON2MtMFl4TzFBMmJrTXB5Mk1YYWU2bmwyWGFBaEVXVXlZS0Zyb3BLaGptTTQzUmlZdS12LUhFdnYzNG1PQnNtdzRYb1BpYlE?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,33 +491,103 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Vulnerabilities</t>
+          <t>Ransomware_Critical_Infra</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+          <t>(ransomware OR "cyber attack") AND ("critical infrastructure" OR "energy sector" OR "power grid" OR "water utility" OR "transport network" OR "financial services" OR "telecoms" OR "government systems") AND (attacked OR disrupted OR warning OR incident OR threat OR advisory)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Critical Microsoft Exchange Server Vulnerability Actively Exploited in Attacks - CyberSecurityNews</t>
+          <t>State-backed ransomware activity raises new concerns over escalating threats to OT, critical infrastructure operations - Industrial Cyber</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sat, 16 May 2026 10:08:55 GMT</t>
+          <t>Sun, 17 May 2026 12:46:44 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOVEVUb05Fbmd1dEdMU2RudVFoV0dHYmMzMS1IMVpFVlNJLUlwMkxOWHhHWEkzLUJtaTV5Vk0tYTFpT1JhU2ZkVXZpNERQNklkYWpLQ3NBLXozNUxuNXZCMTF5VDFHd3RwWjdkQzZFdGlxUzQxVS1yazYxR2hHSWxhWDhISC1tV0HSAYwBQVVfeXFMTjl3RTIxTmVYVGhKSVdEWVBNdHVWT1dFbkdwRkY3OXpNdm5xVC0tRjN1N1k4dWNkNkNneEJxZzlIbHpKamZnYUQ0cGVJaklJWHl1OFRGUzRQQ0tNLWIwdDVGbTFSdDE3WUtaQTJPR2VwQkNoanVTWUNuQnA0SGtKMU9sWVg1ZDk3M0VPb2Q?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOYmFmQ0FRaFhYN0FVMjJoV2s5anJVMUMtaXphVmhaSS0tS1FqRlhZZXJDR09ZU1VRUzNYclpDZHdvbFZGR1FRMjgtcEIzTVg5RnlKTmpqcTlHRHgyanluUjRzOXRVSm52U3VDS3owSjhmWG1hVWJuVnpfaU02NGdDM3pfbFBsV2F6eEd2Z09XNHkteW5GOE9PTXNyaEhxU29ZWEtQQzd4MzZWd1JLUU1GZW4tRzd2Ulg1Q2RMZmR1a2Z1SkhVaUpNenhzbkc3WElVWmVZVzJ5SkRsWmtKcnE0dWhKX0xJQXZGSHc?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ransomware_Groups_New</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lynx attacks on livestock see surge in Chitral - Daily Times</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sun, 17 May 2026 21:50:16 GMT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPcVR5SjVSZ1VYYmRfZzBOYnlYLUtiWnYzdjk5V3NxYzAzMkJ0cjd3V2tQdmpuY3RPZ29XcW12My1uci1EbVdpRGhwOXVUdUZUclI2bE1WSHhLSnhyLWxDLUtKVzZheVM5UEhDUGpxT2c0bl9nQzMtREFLZ1U3TmQxeWZrV3UxVUdC?oc=5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ransomware_Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NGINX CVE-2026-42945 Exploited in the Wild, Causing Worker Crashes and Possible RCE - The Hacker News</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sun, 17 May 2026 11:57:00 GMT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNSV9qTGUzcHVaRTI5TVVWSDU3cU1vQWp0elM5ZGtQcS03SVVvV1RuVnRxZVZoTTVjS2hrN0pvNEp5QmcwV1pWZ055WUs5REhmOUYwc01LYUF5ZVpNWVA3akd2UlFjLVljaEZOUFpmeDJNaF9DTW11TzY5eDFOQm1VZ0RaTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-19 09:31 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Foxconn Suffers Ransomware Attack With Important Project Files From Apple Stolen - ilounge.com</t>
+          <t>News - Zara confirms 200,000 customers’ data exposed in alleged ransomware attack - teiss</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mon, 18 May 2026 04:51:36 GMT</t>
+          <t>Mon, 18 May 2026 23:03:01 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPOG5DelA3dElSaTBEX3ZFV3JRcUV5N1FYbEJtbXpHallOOEVhNF9aXzFzWVhSMjRsM1lyVkZvMjhja3ZVZTBDTHJPTkM0TUg0UXJ3SlNHWFhHWVVRYXRqNnlKc0c1bkxON2MtMFl4TzFBMmJrTXB5Mk1YYWU2bmwyWGFBaEVXVXlZS0Zyb3BLaGptTTQzUmlZdS12LUhFdnYzNG1PQnNtdzRYb1BpYlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPZUpTbjU0M1JJcEl1Y1B0dGloamVRNTl2eW1fZENKbmVLRkdMdDFwcGozNGVJS3NWWEV3ajIwcV9GQjFCTmd2dzZhSDVJekFsejZYRWJrSUY5ZmRzalp4X19sdkplY3phNDJnZ0JGWDRXSDhLTi1Xb29rcnphdk1aTTFkSHg1a0FLY0xfXzllMm1jVVdSUmRtbS1Cc1N3WUkyU3czcEJYS2U0ZjQ?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,27 +491,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Critical_Infra</t>
+          <t>Ransomware_Activity</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(ransomware OR "cyber attack") AND ("critical infrastructure" OR "energy sector" OR "power grid" OR "water utility" OR "transport network" OR "financial services" OR "telecoms" OR "government systems") AND (attacked OR disrupted OR warning OR incident OR threat OR advisory)</t>
+          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>State-backed ransomware activity raises new concerns over escalating threats to OT, critical infrastructure operations - Industrial Cyber</t>
+          <t>Canvas paid hackers: the attack exposed why payment bans ignore operational reality - Cybernews</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sun, 17 May 2026 12:46:44 GMT</t>
+          <t>Mon, 18 May 2026 17:31:20 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOYmFmQ0FRaFhYN0FVMjJoV2s5anJVMUMtaXphVmhaSS0tS1FqRlhZZXJDR09ZU1VRUzNYclpDZHdvbFZGR1FRMjgtcEIzTVg5RnlKTmpqcTlHRHgyanluUjRzOXRVSm52U3VDS3owSjhmWG1hVWJuVnpfaU02NGdDM3pfbFBsV2F6eEd2Z09XNHkteW5GOE9PTXNyaEhxU29ZWEtQQzd4MzZWd1JLUU1GZW4tRzd2Ulg1Q2RMZmR1a2Z1SkhVaUpNenhzbkc3WElVWmVZVzJ5SkRsWmtKcnE0dWhKX0xJQXZGSHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOTkJrS1VyaEhkS3pIWDZ4ajdYYW9OaldvWmcwbFVSWGRoSkNzb05YSlpzT0xOdHM2LXJpOG5jMTlrN0lMTUxCQndkTV9OaURFVVNQNGRocTUwMmxzNnU0VG9zODdQU0hpSExVLVNVOExQWlFweEkyT0tnQWYtM1ZGU2RSTlFHVlU?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -526,27 +526,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ransomware_Groups_New</t>
+          <t>Ransomware_Response</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lynx attacks on livestock see surge in Chitral - Daily Times</t>
+          <t>FBI Newark Seeks Murder Suspect Now Wanted on Federal Charges - Van Nuys News Press</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sun, 17 May 2026 21:50:16 GMT</t>
+          <t>Mon, 18 May 2026 14:45:33 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPcVR5SjVSZ1VYYmRfZzBOYnlYLUtiWnYzdjk5V3NxYzAzMkJ0cjd3V2tQdmpuY3RPZ29XcW12My1uci1EbVdpRGhwOXVUdUZUclI2bE1WSHhLSnhyLWxDLUtKVzZheVM5UEhDUGpxT2c0bl9nQzMtREFLZ1U3TmQxeWZrV3UxVUdC?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOSGlqTjRmSjFXNk41VVpEU2lHSl84T0ZnWGFvRWxlOUluS1hTZl96ZVRZckRhUmszVV9PdUI1T2xZTDFCckVxM0dyLUdzUTgyXy1WdjBrX1JlY3FqRExlbUtaaE9zclJzVEFLT0NkMndqT0llT3ROa19jcGhDbEZub3M5MXY0TXVMMmIxRDNxcVdQOE5nZjJVdWdWcw?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,27 +561,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Vulnerabilities</t>
+          <t>Ransomware_Response</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(vulnerability OR "zero day" OR CVE OR exploit OR patch OR "security flaw" OR "critical flaw") AND (ransomware OR malware OR "threat actor" OR "actively exploited" OR "exploited in the wild" OR "ransomware group") AND (CISA OR advisory OR warning OR alert OR disclosed)</t>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NGINX CVE-2026-42945 Exploited in the Wild, Causing Worker Crashes and Possible RCE - The Hacker News</t>
+          <t>Zeeko Zaki Breaks Silence on ‘FBI’ Season 8 Finale Cliffhanger — Reveals What’s Next for OA - Us Weekly</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sun, 17 May 2026 11:57:00 GMT</t>
+          <t>Tue, 19 May 2026 01:01:39 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNSV9qTGUzcHVaRTI5TVVWSDU3cU1vQWp0elM5ZGtQcS03SVVvV1RuVnRxZVZoTTVjS2hrN0pvNEp5QmcwV1pWZ055WUs5REhmOUYwc01LYUF5ZVpNWVA3akd2UlFjLVljaEZOUFpmeDJNaF9DTW11TzY5eDFOQm1VZ0RaTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPNWRRNEhsUmJqV2trMGN6bUNHQnJRcWEzYlFzV2J4UGNUZjh0R2VOSjQ1cE1vNTlGbmxnOVgyTkpTT3kxQmZfc2RySjJqQjNZNTlaU2NpTWYxYzd2NHZPNWJJNHplTHdBTlQ2WkxaZVRxTFZtaVpSOHdKZUNJYXhyLUhoVlh3dGZ4QjV6c3dVdTNJcTFiQmxBTlhjLTJCdU5abDVhMjF2MWY?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-20 08:58 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>News - Zara confirms 200,000 customers’ data exposed in alleged ransomware attack - teiss</t>
+          <t>AdvancedHEALTH Ransomware Claim Includes 2.3M Patient Data Lines - TechRepublic</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mon, 18 May 2026 23:03:01 GMT</t>
+          <t>Tue, 19 May 2026 13:17:45 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPZUpTbjU0M1JJcEl1Y1B0dGloamVRNTl2eW1fZENKbmVLRkdMdDFwcGozNGVJS3NWWEV3ajIwcV9GQjFCTmd2dzZhSDVJekFsejZYRWJrSUY5ZmRzalp4X19sdkplY3phNDJnZ0JGWDRXSDhLTi1Xb29rcnphdk1aTTFkSHg1a0FLY0xfXzllMm1jVVdSUmRtbS1Cc1N3WUkyU3czcEJYS2U0ZjQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQX05vbE1ZV2hmRWRSVTRiOGpGSFBzVTJhU1BRUkp2X0pJSXNpekRyMDZhVmVBalVXYTVpWlB5TjRTSmpsdjNPU1B5Uzc5MVUtOUZEc2I5aTJnZ0Eyem5HTlpqSE5xNjJlZm9DRWY1MDJvU0o0ckFRQjZtSE9GR250eHpFLU9QUDFyeTVpajJCRVM?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Canvas paid hackers: the attack exposed why payment bans ignore operational reality - Cybernews</t>
+          <t>Liberty Mutual class action claims ransomware attack exposed customer data - Class Action Lawsuits</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mon, 18 May 2026 17:31:20 GMT</t>
+          <t>Tue, 19 May 2026 16:04:35 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOTkJrS1VyaEhkS3pIWDZ4ajdYYW9OaldvWmcwbFVSWGRoSkNzb05YSlpzT0xOdHM2LXJpOG5jMTlrN0lMTUxCQndkTV9OaURFVVNQNGRocTUwMmxzNnU0VG9zODdQU0hpSExVLVNVOExQWlFweEkyT0tnQWYtM1ZGU2RSTlFHVlU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQcDIwb1Jrd005QlpIb09XVWRLNWh5SXVXRU1xWTV0cE5kbWNGTkZ3bE1mTER3SU1xaXJQTzRrV0I0NWpqanp1U09MZTY4UDZhaVg5OVBYSGtyOEtXd0tsa0t2cmI4RU9VUElSQXBYb2tkSXBrZUhlYVFOaHVCTFdoR19JeTlaTlp4Vk9RbVZHOF8wR2Nfb29TN0hNb3pFTmxuRzYxTWJfemZPdi1HX3Bmb19GNUZqQjFrakRaczlGdDNrUjQxaHFWMF9nVjNLRWJNWFE?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -526,27 +526,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ransomware_Response</t>
+          <t>Ransomware_Groups_New</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FBI Newark Seeks Murder Suspect Now Wanted on Federal Charges - Van Nuys News Press</t>
+          <t>UN panel accuses Canadian permanent resident of violating arms embargo on Libya - The Globe and Mail</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mon, 18 May 2026 14:45:33 GMT</t>
+          <t>Tue, 19 May 2026 09:00:00 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOSGlqTjRmSjFXNk41VVpEU2lHSl84T0ZnWGFvRWxlOUluS1hTZl96ZVRZckRhUmszVV9PdUI1T2xZTDFCckVxM0dyLUdzUTgyXy1WdjBrX1JlY3FqRExlbUtaaE9zclJzVEFLT0NkMndqT0llT3ROa19jcGhDbEZub3M5MXY0TXVMMmIxRDNxcVdQOE5nZjJVdWdWcw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQYlMzRjNFNXNoMy02Q0U3MWY0Z0RLX18tbzhJRms5YUxXYWlkVnNuOWQzYU8yLU5VQ0RaeHM1RjNpd1dNemNmQlFWUEtEODl6V2ozUHZzX1Rnak9uVmhac2Jpd20zdHdZOFhfc0NZVFlTbHdSbmgzUUlUMTlfNk95cXBKQlc1NXMxY1c1dC12bHpBbDVHbW1iN0ZXcEI3NU1raXJUUG1OY0MtanBtMG9ISWdlX1R1Zw?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -561,33 +561,103 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ransomware_Response</t>
+          <t>Ransomware_Incidents_UK_EU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+          <t>(ransomware OR "cyber attack" OR "data breach") AND (NHS OR "local council" OR "local authority" OR "public sector" OR university OR school OR manufacturer OR retailer OR "law firm") AND (UK OR Britain OR England OR Scotland OR Wales OR Ireland OR Germany OR France OR Italy OR Spain OR Europe)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Zeeko Zaki Breaks Silence on ‘FBI’ Season 8 Finale Cliffhanger — Reveals What’s Next for OA - Us Weekly</t>
+          <t>M&amp;S profits slide after cyber attack, but retailer hails ‘progress’ - Belfast Telegraph</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tue, 19 May 2026 01:01:39 GMT</t>
+          <t>Wed, 20 May 2026 07:54:48 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPNWRRNEhsUmJqV2trMGN6bUNHQnJRcWEzYlFzV2J4UGNUZjh0R2VOSjQ1cE1vNTlGbmxnOVgyTkpTT3kxQmZfc2RySjJqQjNZNTlaU2NpTWYxYzd2NHZPNWJJNHplTHdBTlQ2WkxaZVRxTFZtaVpSOHdKZUNJYXhyLUhoVlh3dGZ4QjV6c3dVdTNJcTFiQmxBTlhjLTJCdU5abDVhMjF2MWY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPakd5dFYxYWtQQ0ZVaUwzWTRVU3ZoSGs2S0RpRzgwajNVMWNHR0NNMnFsSnlRNU5hSGZMTDFSbXR0Qk9IcW9FWFlxeXJhY25EZHBQWjhadUt4VUp5c2hHRHdTOTd1eFBCUzRPY1J2MVUyYXA0TGdyLVdxN3lUMTB3cXlQZ1F5S0xKMGRpcEdUX3pJdWd4UTk1ZUY1OW12QTVMUy1mUkZLQ2JIQmVYeFBieGRHVzZ0Ql81REs0d0lxaEpad2IwRFQzajJ3QU9kUQ?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Surrey Police investigating child sex abuse allegations after Epstein files release - BBC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tue, 19 May 2026 14:45:30 GMT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1NOFlvaHo3alY2X1lySWlUZWJqczJ1SXRhZ2FGXzZmaWhqcmFYeThCUm0zRm9GS1k1b3Q4cE9QQTI0amxGSUp4NVFqNHBJeUtjeWxNaHprUU9qREZL?oc=5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ransomware_Response</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FBI Offering $500K Reward for Person Of Interest in 2017 Murder of Burlington County Mother and 6-yr-old Son - TAPinto</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tue, 19 May 2026 17:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPcXF1OVpnNWhITXQyNExtUFVRZEF2TndqWHBqd0pGYkNTWEdCdzhIR0RZaGRCbWN3MU9yT0ZtSjdlejRqcGYzVUFDak1IRjB2d2ktajEtNHhQU1VDZnhxR3R0cTNPSHR6M2xXOWtYcXNWazZjenFHR0tXVGxnWGxiTVVkYjFXbk9hWTF3MG1vRGptRVE3VW9Gem05THVuYlNFdnRObEpQYUZJWUhyWWEwWXVCVWRSTTYwMjBISlc0MFhWRVJKOTFhYVlYbUxKdEdlV3RCZzN3MHBkcVJfU0pQVWxZOUV0dGYzTUVhT1M4ZXdxaEFnV045endNVll6Um1Mb0FyWjNaS0FpZ1VpS2hwRmVB?oc=5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>

<commit_message>
Ransomware feed update — 2026-05-21 09:01 UTC
</commit_message>
<xml_diff>
--- a/data/ransomware_latest.xlsx
+++ b/data/ransomware_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AdvancedHEALTH Ransomware Claim Includes 2.3M Patient Data Lines - TechRepublic</t>
+          <t>Minnesota school cancels classes over ransomware attack - CBS News</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 19 May 2026 13:17:45 GMT</t>
+          <t>Wed, 20 May 2026 23:52:00 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQX05vbE1ZV2hmRWRSVTRiOGpGSFBzVTJhU1BRUkp2X0pJSXNpekRyMDZhVmVBalVXYTVpWlB5TjRTSmpsdjNPU1B5Uzc5MVUtOUZEc2I5aTJnZ0Eyem5HTlpqSE5xNjJlZm9DRWY1MDJvU0o0ckFRQjZtSE9GR250eHpFLU9QUDFyeTVpajJCRVM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQZzVUTGhJYldGSE1GenUwNnNyV1hkY1pFa0FnSkdEZjVrUWhHTmJKVF9pM1ZMYTBhcjA1MlFScFQyRDNzM1lCVGR3UVdHWWJBWXJlZnp6UmtnU0pxUHNubk1fZURzTmwtVXgtb0N5c3dPTzRUMFl1ZVFEcUFiUzRINEs2RzZhbkl5akdhUUV1WWhaVFlrZHY1UkJTeEc?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -491,173 +491,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ransomware_Activity</t>
+          <t>Ransomware_Response</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("LockBit" OR "ALPHV" OR "RansomHub" OR "Akira" OR "Black Basta" OR "Cl0p" OR "Medusa" OR "Scattered Spider" OR "DragonForce" OR "8Base" OR "ShinyHunters" OR "ransomware attack" OR "ransomware incident" OR "ransom demand" OR "data encrypted" OR "systems encrypted") AND (attack OR victim OR hospital OR government OR company OR "critical infrastructure" OR UK OR Europe OR "United States" OR disclosed OR confirmed)</t>
+          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Liberty Mutual class action claims ransomware attack exposed customer data - Class Action Lawsuits</t>
+          <t>Nancy Guthrie abduction: FBI analyzing DNA recovered from her home, sources say - ABC11 Raleigh-Durham</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tue, 19 May 2026 16:04:35 GMT</t>
+          <t>Wed, 20 May 2026 10:41:19 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQcDIwb1Jrd005QlpIb09XVWRLNWh5SXVXRU1xWTV0cE5kbWNGTkZ3bE1mTER3SU1xaXJQTzRrV0I0NWpqanp1U09MZTY4UDZhaVg5OVBYSGtyOEtXd0tsa0t2cmI4RU9VUElSQXBYb2tkSXBrZUhlYVFOaHVCTFdoR19JeTlaTlp4Vk9RbVZHOF8wR2Nfb29TN0hNb3pFTmxuRzYxTWJfemZPdi1HX3Bmb19GNUZqQjFrakRaczlGdDNrUjQxaHFWMF9nVjNLRWJNWFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixANBVV95cUxOSzl6M3V6NUl4aWdNbDhBYlJTdUx3TWdjSmRXdnRrM0M4dzhMeHdzMHB2Z1RqOWY5UjIwR1U0YzhZOUhmYlNsVGQyZU1kckdwdG5tNGJYYlRFcTFhUFozS0FvcElyVlpZS3cwTnB3MEo4MEtiTWVMbDE4VWlPWDNiX213RWZkZS1jNS0wTGtqWGFTUTlwSVU4c3FIZUxiWVd6MzN3bXNFYTh0RFdlSVpqVGUzc2ZtVkgzQ1N1eERtd1lxWXBPaG9JNzZxbDdkVENKMXFfQVI5QmpwdGp2VkRxYm5MbVNxa2RIWW9nOTFVZldZT2YxVEtTR29vZUpDdFVPM20tUGI2YUpLYW51alM2ekxob09FODdhZWFlZmZZeGk3aWo1TVBJd21ZMmFMdXp4cXFlRTdzSVhLSFl1TGJhZ01oYjEwb2x4cUVvSjFIeFpLazg3NkhMaHR0c2JTS1BWUEdEbDZ5UGxhVmlacGtPSTZ0di1jTm9fbjhSc1RacVpYWDgzN1FDSTNFLTRiRGpuVGhUT2NpZEUyUS1NX1pHaURPM2paNk1BaVVTM0ZNTFVDaGIwcGg3VFloZ2ttRHVVTFhyaA?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ransomware_Groups_New</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>("BlackSuit" OR "Hunters International" OR "Qilin" OR "INC Ransom" OR "Rhysida" OR "NoEscape" OR "Cactus" OR "Meow" OR "Embargo" OR "Fog" OR "Interlock" OR "SafePay" OR "Lynx" OR "Cicada3301" OR "RansomedVC") AND (attack OR victim OR campaign OR active OR claimed OR leaked OR posted OR operation OR arrested)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>UN panel accuses Canadian permanent resident of violating arms embargo on Libya - The Globe and Mail</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Tue, 19 May 2026 09:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQYlMzRjNFNXNoMy02Q0U3MWY0Z0RLX18tbzhJRms5YUxXYWlkVnNuOWQzYU8yLU5VQ0RaeHM1RjNpd1dNemNmQlFWUEtEODl6V2ozUHZzX1Rnak9uVmhac2Jpd20zdHdZOFhfc0NZVFlTbHdSbmgzUUlUMTlfNk95cXBKQlc1NXMxY1c1dC12bHpBbDVHbW1iN0ZXcEI3NU1raXJUUG1OY0MtanBtMG9ISWdlX1R1Zw?oc=5</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ransomware_Incidents_UK_EU</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>(ransomware OR "cyber attack" OR "data breach") AND (NHS OR "local council" OR "local authority" OR "public sector" OR university OR school OR manufacturer OR retailer OR "law firm") AND (UK OR Britain OR England OR Scotland OR Wales OR Ireland OR Germany OR France OR Italy OR Spain OR Europe)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>M&amp;S profits slide after cyber attack, but retailer hails ‘progress’ - Belfast Telegraph</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Wed, 20 May 2026 07:54:48 GMT</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPakd5dFYxYWtQQ0ZVaUwzWTRVU3ZoSGs2S0RpRzgwajNVMWNHR0NNMnFsSnlRNU5hSGZMTDFSbXR0Qk9IcW9FWFlxeXJhY25EZHBQWjhadUt4VUp5c2hHRHdTOTd1eFBCUzRPY1J2MVUyYXA0TGdyLVdxN3lUMTB3cXlQZ1F5S0xKMGRpcEdUX3pJdWd4UTk1ZUY1OW12QTVMUy1mUkZLQ2JIQmVYeFBieGRHVzZ0Ql81REs0d0lxaEpad2IwRFQzajJ3QU9kUQ?oc=5</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ransomware_Response</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Surrey Police investigating child sex abuse allegations after Epstein files release - BBC</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Tue, 19 May 2026 14:45:30 GMT</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1NOFlvaHo3alY2X1lySWlUZWJqczJ1SXRhZ2FGXzZmaWhqcmFYeThCUm0zRm9GS1k1b3Q4cE9QQTI0amxGSUp4NVFqNHBJeUtjeWxNaHprUU9qREZL?oc=5</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ransomware_Response</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>(Europol OR FBI OR "National Crime Agency" OR CISA OR "Department of Justice" OR Interpol OR "ransomware arrest" OR "hacker indicted" OR "cybercriminal arrested" OR "ransomware gang arrested" OR "ransomware operator charged" OR "ransomware infrastructure seized" OR "cyber operation dismantled" OR "ransomware advisory" OR "mitigation guidance") AND (ransomware OR cybercrime OR "cyber criminal" OR "threat actor" OR "ransomware gang" OR malware)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>FBI Offering $500K Reward for Person Of Interest in 2017 Murder of Burlington County Mother and 6-yr-old Son - TAPinto</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Tue, 19 May 2026 17:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikgJBVV95cUxPcXF1OVpnNWhITXQyNExtUFVRZEF2TndqWHBqd0pGYkNTWEdCdzhIR0RZaGRCbWN3MU9yT0ZtSjdlejRqcGYzVUFDak1IRjB2d2ktajEtNHhQU1VDZnhxR3R0cTNPSHR6M2xXOWtYcXNWazZjenFHR0tXVGxnWGxiTVVkYjFXbk9hWTF3MG1vRGptRVE3VW9Gem05THVuYlNFdnRObEpQYUZJWUhyWWEwWXVCVWRSTTYwMjBISlc0MFhWRVJKOTFhYVlYbUxKdEdlV3RCZzN3MHBkcVJfU0pQVWxZOUV0dGYzTUVhT1M4ZXdxaEFnV045endNVll6Um1Mb0FyWjNaS0FpZ1VpS2hwRmVB?oc=5</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>google_rss</t>
         </is>

</xml_diff>